<commit_message>
Actualizacion semanal automatica 2026-05-23
</commit_message>
<xml_diff>
--- a/Acervo_Jurisprudencial.xlsx
+++ b/Acervo_Jurisprudencial.xlsx
@@ -20,12 +20,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Penal" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acervo (maestra)'!$A$1:$V$108</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Administrativo'!$A$1:$V$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Acervo (maestra)'!$A$1:$V$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Administrativo'!$A$1:$V$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Amparo'!$A$1:$V$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Civil'!$A$1:$V$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Civil — Condominio'!$A$1:$V$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Constitucional - DDHH'!$A$1:$V$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Constitucional - DDHH'!$A$1:$V$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Fiscal'!$A$1:$V$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Laboral'!$A$1:$V$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Mercantil'!$A$1:$V$13</definedName>
@@ -635,27 +635,27 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Penal</t>
+          <t>Constitucional / DDHH</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Constitucional / DDHH</t>
+          <t>Penal</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Mercantil</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
@@ -665,11 +665,11 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Administrativo</t>
+          <t>Mercantil</t>
         </is>
       </c>
       <c r="B20" s="8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="21">
@@ -768,7 +768,7 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -3654,7 +3654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V108"/>
+  <dimension ref="A1:V111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10304,7 +10304,7 @@
     <row r="72" ht="80" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>amp-eje-001</t>
+          <t>auto-2032177</t>
         </is>
       </c>
       <c r="B72" s="11" t="n">
@@ -10317,17 +10317,17 @@
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>Amparo</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>Amparo contra normas generales</t>
+          <t>Responsabilidad administrativa de servidores públicos</t>
         </is>
       </c>
       <c r="F72" s="11" t="inlineStr">
         <is>
-          <t>Efectos reflejos del fallo</t>
+          <t>Actualización automática semanal</t>
         </is>
       </c>
       <c r="G72" s="11" t="inlineStr">
@@ -10337,7 +10337,7 @@
       </c>
       <c r="H72" s="11" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
@@ -10352,57 +10352,57 @@
       </c>
       <c r="K72" s="12" t="inlineStr">
         <is>
-          <t>AMPARO CONTRA NORMAS GENERALES. SU NEGATIVA VINCULA Y TIENE EFECTOS REFLEJOS EN OTROS LITIGIOS DONDE LA MISMA PERSONA SOLICITE, EN EJERCICIO DEL CONTROL DIFUSO O DE CONSTITUCIONALIDAD Y CONVENCIONALIDAD EX OFFICIO, LA INAPLICACIÓN DE AQUÉLLAS.</t>
+          <t>PRUEBAS EN EL JUICIO CONTENCIOSO ADMINISTRATIVO FEDERAL. EL ARTÍCULO 40, PÁRRAFO SEGUNDO, DE LA LEY FEDERAL DE PROCEDIMIENTO CONTENCIOSO ADMINISTRATIVO NO VIOLA EL DERECHO DE ACCESO A LA JUSTICIA.</t>
         </is>
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>2029745</t>
+          <t>2032177</t>
         </is>
       </c>
       <c r="M72" s="11" t="inlineStr"/>
       <c r="N72" s="11" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
         </is>
       </c>
       <c r="O72" s="11" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — captura automática</t>
         </is>
       </c>
       <c r="P72" s="11" t="inlineStr"/>
       <c r="Q72" s="11" t="inlineStr">
         <is>
-          <t>Si una persona pierde amparo contra norma general, esa cosa juzgada le aplica también en otros litigios donde pretenda inaplicación de la misma norma por control difuso.</t>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
         </is>
       </c>
       <c r="R72" s="11" t="inlineStr">
         <is>
-          <t>Cierra puerta a relitigar inconstitucionalidad por vías paralelas.</t>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
         </is>
       </c>
       <c r="S72" s="11" t="inlineStr">
         <is>
-          <t>Si ya perdiste amparo contra norma, no insistas vía control difuso en otro juicio.</t>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
         </is>
       </c>
       <c r="T72" s="11" t="inlineStr"/>
       <c r="U72" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029745</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032177</t>
         </is>
       </c>
       <c r="V72" s="11" t="inlineStr">
         <is>
-          <t>amparo normas · control difuso · efectos reflejos</t>
+          <t>Responsabilidad administrativa de servidores públicos · actualización automática</t>
         </is>
       </c>
     </row>
     <row r="73" ht="80" customHeight="1">
       <c r="A73" s="13" t="inlineStr">
         <is>
-          <t>amp-sus-002</t>
+          <t>amp-eje-001</t>
         </is>
       </c>
       <c r="B73" s="13" t="n">
@@ -10420,12 +10420,12 @@
       </c>
       <c r="E73" s="13" t="inlineStr">
         <is>
-          <t>Suspensión</t>
+          <t>Amparo contra normas generales</t>
         </is>
       </c>
       <c r="F73" s="13" t="inlineStr">
         <is>
-          <t>Suspensión contra medidas cautelares civiles/mercantiles</t>
+          <t>Efectos reflejos del fallo</t>
         </is>
       </c>
       <c r="G73" s="13" t="inlineStr">
@@ -10435,7 +10435,7 @@
       </c>
       <c r="H73" s="13" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I73" s="13" t="inlineStr">
@@ -10450,57 +10450,57 @@
       </c>
       <c r="K73" s="14" t="inlineStr">
         <is>
-          <t>SUSPENSIÓN EN EL JUICIO DE AMPARO. PUEDE CONCEDERSE CONTRA MEDIDAS CAUTELARES DICTADAS EN PROCESOS CIVILES O MERCANTILES CUANDO NO PRESERVAN LA MATERIA DEL JUICIO DE ORIGEN O IMPONEN RESTRICCIONES GENÉRICAS QUE AFECTAN INJUSTIFICADAMENTE DERECHOS HUMANOS.</t>
+          <t>AMPARO CONTRA NORMAS GENERALES. SU NEGATIVA VINCULA Y TIENE EFECTOS REFLEJOS EN OTROS LITIGIOS DONDE LA MISMA PERSONA SOLICITE, EN EJERCICIO DEL CONTROL DIFUSO O DE CONSTITUCIONALIDAD Y CONVENCIONALIDAD EX OFFICIO, LA INAPLICACIÓN DE AQUÉLLAS.</t>
         </is>
       </c>
       <c r="L73" s="13" t="inlineStr">
         <is>
-          <t>2032118</t>
+          <t>2029745</t>
         </is>
       </c>
       <c r="M73" s="13" t="inlineStr"/>
       <c r="N73" s="13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="O73" s="13" t="inlineStr">
         <is>
-          <t>SJF 12a Época — VERIFICADO</t>
+          <t>Gaceta SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P73" s="13" t="inlineStr"/>
       <c r="Q73" s="13" t="inlineStr">
         <is>
-          <t>Las medidas cautelares civiles o mercantiles (embargos, restricciones, prohibiciones) pueden suspenderse vía amparo si exceden lo necesario para preservar la materia o son genéricas y afectan derechos humanos.</t>
+          <t>Si una persona pierde amparo contra norma general, esa cosa juzgada le aplica también en otros litigios donde pretenda inaplicación de la misma norma por control difuso.</t>
         </is>
       </c>
       <c r="R73" s="13" t="inlineStr">
         <is>
-          <t>Defensa contra embargos abusivos y medidas precautorias excesivas.</t>
+          <t>Cierra puerta a relitigar inconstitucionalidad por vías paralelas.</t>
         </is>
       </c>
       <c r="S73" s="13" t="inlineStr">
         <is>
-          <t>Embargado puede amparar si la medida es desproporcionada o no preserva materia del juicio.</t>
+          <t>Si ya perdiste amparo contra norma, no insistas vía control difuso en otro juicio.</t>
         </is>
       </c>
       <c r="T73" s="13" t="inlineStr"/>
       <c r="U73" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032118</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029745</t>
         </is>
       </c>
       <c r="V73" s="13" t="inlineStr">
         <is>
-          <t>suspensión amparo · medida cautelar · 12a Época</t>
+          <t>amparo normas · control difuso · efectos reflejos</t>
         </is>
       </c>
     </row>
     <row r="74" ht="80" customHeight="1">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>amp-sus-003</t>
+          <t>amp-sus-002</t>
         </is>
       </c>
       <c r="B74" s="11" t="n">
@@ -10523,7 +10523,7 @@
       </c>
       <c r="F74" s="11" t="inlineStr">
         <is>
-          <t>Suspensión con efectos restitutorios — incapacidad médica</t>
+          <t>Suspensión contra medidas cautelares civiles/mercantiles</t>
         </is>
       </c>
       <c r="G74" s="11" t="inlineStr">
@@ -10548,12 +10548,12 @@
       </c>
       <c r="K74" s="12" t="inlineStr">
         <is>
-          <t>SUSPENSIÓN EN AMPARO INDIRECTO CON EFECTOS RESTITUTORIOS. PROCEDE PARA LA EXPEDICIÓN DE UNA INCAPACIDAD MÉDICA CUANDO SU EFECTO ES TRANSITORIO Y EXISTE UN ESTADO CLÍNICO INCAPACITANTE PREVIAMENTE ACREDITADO.</t>
+          <t>SUSPENSIÓN EN EL JUICIO DE AMPARO. PUEDE CONCEDERSE CONTRA MEDIDAS CAUTELARES DICTADAS EN PROCESOS CIVILES O MERCANTILES CUANDO NO PRESERVAN LA MATERIA DEL JUICIO DE ORIGEN O IMPONEN RESTRICCIONES GENÉRICAS QUE AFECTAN INJUSTIFICADAMENTE DERECHOS HUMANOS.</t>
         </is>
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>2032066</t>
+          <t>2032118</t>
         </is>
       </c>
       <c r="M74" s="11" t="inlineStr"/>
@@ -10570,35 +10570,35 @@
       <c r="P74" s="11" t="inlineStr"/>
       <c r="Q74" s="11" t="inlineStr">
         <is>
-          <t>La suspensión puede tener efectos restitutorios (no solo conservativos): obligar al IMSS/ISSSTE a expedir incapacidad médica si hay estado clínico acreditado.</t>
+          <t>Las medidas cautelares civiles o mercantiles (embargos, restricciones, prohibiciones) pueden suspenderse vía amparo si exceden lo necesario para preservar la materia o son genéricas y afectan derechos humanos.</t>
         </is>
       </c>
       <c r="R74" s="11" t="inlineStr">
         <is>
-          <t>Innovadora: suspensión que ORDENA actuar, no solo paraliza.</t>
+          <t>Defensa contra embargos abusivos y medidas precautorias excesivas.</t>
         </is>
       </c>
       <c r="S74" s="11" t="inlineStr">
         <is>
-          <t>Útil para trabajadores cuyas incapacidades son negadas pese a sustento médico.</t>
+          <t>Embargado puede amparar si la medida es desproporcionada o no preserva materia del juicio.</t>
         </is>
       </c>
       <c r="T74" s="11" t="inlineStr"/>
       <c r="U74" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032066</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032118</t>
         </is>
       </c>
       <c r="V74" s="11" t="inlineStr">
         <is>
-          <t>suspensión restitutoria · incapacidad médica · IMSS · 12a Época</t>
+          <t>suspensión amparo · medida cautelar · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="75" ht="80" customHeight="1">
       <c r="A75" s="13" t="inlineStr">
         <is>
-          <t>civ-arr-003</t>
+          <t>amp-sus-003</t>
         </is>
       </c>
       <c r="B75" s="13" t="n">
@@ -10611,17 +10611,17 @@
       </c>
       <c r="D75" s="13" t="inlineStr">
         <is>
-          <t>Civil</t>
+          <t>Amparo</t>
         </is>
       </c>
       <c r="E75" s="13" t="inlineStr">
         <is>
-          <t>Arrendamiento</t>
+          <t>Suspensión</t>
         </is>
       </c>
       <c r="F75" s="13" t="inlineStr">
         <is>
-          <t>Tácita reconducción</t>
+          <t>Suspensión con efectos restitutorios — incapacidad médica</t>
         </is>
       </c>
       <c r="G75" s="13" t="inlineStr">
@@ -10631,7 +10631,7 @@
       </c>
       <c r="H75" s="13" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I75" s="13" t="inlineStr">
@@ -10641,54 +10641,62 @@
       </c>
       <c r="J75" s="13" t="inlineStr">
         <is>
-          <t>Federal — interpreta CCCDMX</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K75" s="14" t="inlineStr">
         <is>
-          <t>TÁCITA RECONDUCCIÓN DEL ARRENDAMIENTO. SUS REQUISITOS Y EFECTOS CONFORME AL CÓDIGO CIVIL PARA EL DISTRITO FEDERAL.</t>
+          <t>SUSPENSIÓN EN AMPARO INDIRECTO CON EFECTOS RESTITUTORIOS. PROCEDE PARA LA EXPEDICIÓN DE UNA INCAPACIDAD MÉDICA CUANDO SU EFECTO ES TRANSITORIO Y EXISTE UN ESTADO CLÍNICO INCAPACITANTE PREVIAMENTE ACREDITADO.</t>
         </is>
       </c>
       <c r="L75" s="13" t="inlineStr">
         <is>
-          <t>2017872</t>
+          <t>2032066</t>
         </is>
       </c>
       <c r="M75" s="13" t="inlineStr"/>
-      <c r="N75" s="13" t="inlineStr"/>
-      <c r="O75" s="13" t="inlineStr"/>
+      <c r="N75" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="O75" s="13" t="inlineStr">
+        <is>
+          <t>SJF 12a Época — VERIFICADO</t>
+        </is>
+      </c>
       <c r="P75" s="13" t="inlineStr"/>
       <c r="Q75" s="13" t="inlineStr">
         <is>
-          <t>Vencido el contrato, si el arrendatario continúa en la posesión del bien con consentimiento del arrendador (recibos de renta o silencio) por más de 10 días, el contrato se considera renovado por tiempo indeterminado.</t>
+          <t>La suspensión puede tener efectos restitutorios (no solo conservativos): obligar al IMSS/ISSSTE a expedir incapacidad médica si hay estado clínico acreditado.</t>
         </is>
       </c>
       <c r="R75" s="13" t="inlineStr">
         <is>
-          <t>Trampa frecuente: el arrendador pierde plazo fijo por no actuar.</t>
+          <t>Innovadora: suspensión que ORDENA actuar, no solo paraliza.</t>
         </is>
       </c>
       <c r="S75" s="13" t="inlineStr">
         <is>
-          <t>Al vencer el contrato, el arrendador debe requerir formalmente desocupación si no quiere renovación tácita. Recibir un solo pago posterior al vencimiento es indicio fuerte de reconducción.</t>
+          <t>Útil para trabajadores cuyas incapacidades son negadas pese a sustento médico.</t>
         </is>
       </c>
       <c r="T75" s="13" t="inlineStr"/>
       <c r="U75" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2017872</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032066</t>
         </is>
       </c>
       <c r="V75" s="13" t="inlineStr">
         <is>
-          <t>tácita reconducción · vencimiento · renovación</t>
+          <t>suspensión restitutoria · incapacidad médica · IMSS · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="76" ht="80" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>civ-arr-004</t>
+          <t>civ-arr-003</t>
         </is>
       </c>
       <c r="B76" s="11" t="n">
@@ -10711,7 +10719,7 @@
       </c>
       <c r="F76" s="11" t="inlineStr">
         <is>
-          <t>Consignación de llaves no libera de pago</t>
+          <t>Tácita reconducción</t>
         </is>
       </c>
       <c r="G76" s="11" t="inlineStr">
@@ -10721,7 +10729,7 @@
       </c>
       <c r="H76" s="11" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
@@ -10731,62 +10739,54 @@
       </c>
       <c r="J76" s="11" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Federal — interpreta CCCDMX</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr">
         <is>
-          <t>ARRENDAMIENTO. LA CONSIGNACIÓN DE LLAVES DEL INMUEBLE ARRENDADO EXHIBIDAS MEDIANTE ESCRITO ANTE EL ÓRGANO JURISDICCIONAL NO LIBERA AL DEMANDADO DEL PAGO DE RENTAS, MANTENIMIENTO, SERVICIOS DE GAS Y AGUA, SI NO ACREDITA HABER IMPULSADO EL PROCEDIMIENTO.</t>
+          <t>TÁCITA RECONDUCCIÓN DEL ARRENDAMIENTO. SUS REQUISITOS Y EFECTOS CONFORME AL CÓDIGO CIVIL PARA EL DISTRITO FEDERAL.</t>
         </is>
       </c>
       <c r="L76" s="11" t="inlineStr">
         <is>
-          <t>2031626</t>
+          <t>2017872</t>
         </is>
       </c>
       <c r="M76" s="11" t="inlineStr"/>
-      <c r="N76" s="11" t="inlineStr">
-        <is>
-          <t>2025-2026</t>
-        </is>
-      </c>
-      <c r="O76" s="11" t="inlineStr">
-        <is>
-          <t>Semanario Judicial de la Federación — VERIFICADO</t>
-        </is>
-      </c>
+      <c r="N76" s="11" t="inlineStr"/>
+      <c r="O76" s="11" t="inlineStr"/>
       <c r="P76" s="11" t="inlineStr"/>
       <c r="Q76" s="11" t="inlineStr">
         <is>
-          <t>El arrendatario que pretende terminar el contrato consignando las llaves debe impulsar la notificación al arrendador. Sin ese impulso procesal, sigue obligado al pago de rentas y servicios.</t>
+          <t>Vencido el contrato, si el arrendatario continúa en la posesión del bien con consentimiento del arrendador (recibos de renta o silencio) por más de 10 días, el contrato se considera renovado por tiempo indeterminado.</t>
         </is>
       </c>
       <c r="R76" s="11" t="inlineStr">
         <is>
-          <t>Defensa del arrendador contra inquilinos que abandonan sin notificar.</t>
+          <t>Trampa frecuente: el arrendador pierde plazo fijo por no actuar.</t>
         </is>
       </c>
       <c r="S76" s="11" t="inlineStr">
         <is>
-          <t>Inquilino que entrega llaves debe pedir actuario para notificar, no basta exhibirlas. Arrendador puede seguir cobrando hasta que el procedimiento esté impulsado.</t>
+          <t>Al vencer el contrato, el arrendador debe requerir formalmente desocupación si no quiere renovación tácita. Recibir un solo pago posterior al vencimiento es indicio fuerte de reconducción.</t>
         </is>
       </c>
       <c r="T76" s="11" t="inlineStr"/>
       <c r="U76" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031626</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2017872</t>
         </is>
       </c>
       <c r="V76" s="11" t="inlineStr">
         <is>
-          <t>arrendamiento · consignación llaves · 12a Época</t>
+          <t>tácita reconducción · vencimiento · renovación</t>
         </is>
       </c>
     </row>
     <row r="77" ht="80" customHeight="1">
       <c r="A77" s="13" t="inlineStr">
         <is>
-          <t>civ-arr-005</t>
+          <t>civ-arr-004</t>
         </is>
       </c>
       <c r="B77" s="13" t="n">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="F77" s="13" t="inlineStr">
         <is>
-          <t>Aviso de terminación — cómputo de plazo</t>
+          <t>Consignación de llaves no libera de pago</t>
         </is>
       </c>
       <c r="G77" s="13" t="inlineStr">
@@ -10819,7 +10819,7 @@
       </c>
       <c r="H77" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I77" s="13" t="inlineStr">
@@ -10829,62 +10829,62 @@
       </c>
       <c r="J77" s="13" t="inlineStr">
         <is>
-          <t>CDMX</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K77" s="14" t="inlineStr">
         <is>
-          <t>CONTRATO DE ARRENDAMIENTO POR TIEMPO INDETERMINADO PARA PREDIOS URBANOS. LA OPORTUNIDAD DEL AVISO PARA DARLO POR CONCLUIDO DEBE COMPUTARSE EN DÍAS HÁBILES, A MENOS QUE LAS PARTES RENUNCIEN A ESE DERECHO.</t>
+          <t>ARRENDAMIENTO. LA CONSIGNACIÓN DE LLAVES DEL INMUEBLE ARRENDADO EXHIBIDAS MEDIANTE ESCRITO ANTE EL ÓRGANO JURISDICCIONAL NO LIBERA AL DEMANDADO DEL PAGO DE RENTAS, MANTENIMIENTO, SERVICIOS DE GAS Y AGUA, SI NO ACREDITA HABER IMPULSADO EL PROCEDIMIENTO.</t>
         </is>
       </c>
       <c r="L77" s="13" t="inlineStr">
         <is>
-          <t>2024563</t>
+          <t>2031626</t>
         </is>
       </c>
       <c r="M77" s="13" t="inlineStr"/>
       <c r="N77" s="13" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O77" s="13" t="inlineStr">
         <is>
-          <t>Gaceta del SJF — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — VERIFICADO</t>
         </is>
       </c>
       <c r="P77" s="13" t="inlineStr"/>
       <c r="Q77" s="13" t="inlineStr">
         <is>
-          <t>El aviso de terminación de arrendamiento por tiempo indeterminado se computa en días HÁBILES por defecto. Solo si las partes pactaron expresamente días naturales, aplica esa modalidad.</t>
+          <t>El arrendatario que pretende terminar el contrato consignando las llaves debe impulsar la notificación al arrendador. Sin ese impulso procesal, sigue obligado al pago de rentas y servicios.</t>
         </is>
       </c>
       <c r="R77" s="13" t="inlineStr">
         <is>
-          <t>Define plazo real para desocupación en CDMX.</t>
+          <t>Defensa del arrendador contra inquilinos que abandonan sin notificar.</t>
         </is>
       </c>
       <c r="S77" s="13" t="inlineStr">
         <is>
-          <t>Confusión frecuente: muchos contratos asumen días naturales sin pactarlo. El plazo es hábil. Hay que dar el aviso anticipándose.</t>
+          <t>Inquilino que entrega llaves debe pedir actuario para notificar, no basta exhibirlas. Arrendador puede seguir cobrando hasta que el procedimiento esté impulsado.</t>
         </is>
       </c>
       <c r="T77" s="13" t="inlineStr"/>
       <c r="U77" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024563</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031626</t>
         </is>
       </c>
       <c r="V77" s="13" t="inlineStr">
         <is>
-          <t>arrendamiento CDMX · aviso terminación · días hábiles</t>
+          <t>arrendamiento · consignación llaves · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="78" ht="80" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>fam-div-001</t>
+          <t>civ-arr-005</t>
         </is>
       </c>
       <c r="B78" s="11" t="n">
@@ -10902,12 +10902,12 @@
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>Divorcio sin expresión de causa</t>
+          <t>Arrendamiento</t>
         </is>
       </c>
       <c r="F78" s="11" t="inlineStr">
         <is>
-          <t>Procedencia del recurso de revocación</t>
+          <t>Aviso de terminación — cómputo de plazo</t>
         </is>
       </c>
       <c r="G78" s="11" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="H78" s="11" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I78" s="11" t="inlineStr">
@@ -10932,57 +10932,57 @@
       </c>
       <c r="K78" s="12" t="inlineStr">
         <is>
-          <t>DIVORCIO SIN EXPRESIÓN DE CAUSA. PROCEDENCIA DEL RECURSO DE REVOCACIÓN CONTRA LAS RESOLUCIONES DICTADAS DURANTE SU SUSTANCIACIÓN.</t>
+          <t>CONTRATO DE ARRENDAMIENTO POR TIEMPO INDETERMINADO PARA PREDIOS URBANOS. LA OPORTUNIDAD DEL AVISO PARA DARLO POR CONCLUIDO DEBE COMPUTARSE EN DÍAS HÁBILES, A MENOS QUE LAS PARTES RENUNCIEN A ESE DERECHO.</t>
         </is>
       </c>
       <c r="L78" s="11" t="inlineStr">
         <is>
-          <t>2031170</t>
+          <t>2024563</t>
         </is>
       </c>
       <c r="M78" s="11" t="inlineStr"/>
       <c r="N78" s="11" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="O78" s="11" t="inlineStr">
         <is>
-          <t>SJF — VERIFICADO</t>
+          <t>Gaceta del SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P78" s="11" t="inlineStr"/>
       <c r="Q78" s="11" t="inlineStr">
         <is>
-          <t>Las resoluciones dictadas durante la sustanciación del divorcio sin causa admiten recurso de revocación conforme a los arts. 685, 685 bis y 691 del CPC para CDMX.</t>
+          <t>El aviso de terminación de arrendamiento por tiempo indeterminado se computa en días HÁBILES por defecto. Solo si las partes pactaron expresamente días naturales, aplica esa modalidad.</t>
         </is>
       </c>
       <c r="R78" s="11" t="inlineStr">
         <is>
-          <t>Vía expedita contra resoluciones intermedias en divorcio incausado CDMX.</t>
+          <t>Define plazo real para desocupación en CDMX.</t>
         </is>
       </c>
       <c r="S78" s="11" t="inlineStr">
         <is>
-          <t>Antes era confusa la vía. Ahora con esta tesis se aplica revocación. Permite revisar rápidamente medidas provisionales sobre alimentos o convivencia.</t>
+          <t>Confusión frecuente: muchos contratos asumen días naturales sin pactarlo. El plazo es hábil. Hay que dar el aviso anticipándose.</t>
         </is>
       </c>
       <c r="T78" s="11" t="inlineStr"/>
       <c r="U78" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031170</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024563</t>
         </is>
       </c>
       <c r="V78" s="11" t="inlineStr">
         <is>
-          <t>divorcio incausado · revocación · CDMX · 12a Época</t>
+          <t>arrendamiento CDMX · aviso terminación · días hábiles</t>
         </is>
       </c>
     </row>
     <row r="79" ht="80" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
         <is>
-          <t>fam-div-002</t>
+          <t>fam-div-001</t>
         </is>
       </c>
       <c r="B79" s="13" t="n">
@@ -11005,7 +11005,7 @@
       </c>
       <c r="F79" s="13" t="inlineStr">
         <is>
-          <t>Amparo directo contra sentencia</t>
+          <t>Procedencia del recurso de revocación</t>
         </is>
       </c>
       <c r="G79" s="13" t="inlineStr">
@@ -11015,7 +11015,7 @@
       </c>
       <c r="H79" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I79" s="13" t="inlineStr">
@@ -11025,23 +11025,23 @@
       </c>
       <c r="J79" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>CDMX</t>
         </is>
       </c>
       <c r="K79" s="14" t="inlineStr">
         <is>
-          <t>AMPARO DIRECTO. PROCEDE CONTRA LA SENTENCIA QUE DECLARA LA DISOLUCIÓN DEL VÍNCULO MATRIMONIAL EN UN JUICIO DE DIVORCIO SIN EXPRESIÓN DE CAUSA Y RESUELVE PROVISIONALMENTE SOBRE LOS ALIMENTOS U OTRAS CUESTIONES INHERENTES.</t>
+          <t>DIVORCIO SIN EXPRESIÓN DE CAUSA. PROCEDENCIA DEL RECURSO DE REVOCACIÓN CONTRA LAS RESOLUCIONES DICTADAS DURANTE SU SUSTANCIACIÓN.</t>
         </is>
       </c>
       <c r="L79" s="13" t="inlineStr">
         <is>
-          <t>2029853</t>
+          <t>2031170</t>
         </is>
       </c>
       <c r="M79" s="13" t="inlineStr"/>
       <c r="N79" s="13" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O79" s="13" t="inlineStr">
@@ -11052,35 +11052,35 @@
       <c r="P79" s="13" t="inlineStr"/>
       <c r="Q79" s="13" t="inlineStr">
         <is>
-          <t>La sentencia de divorcio sin expresión de causa que resuelve sobre alimentos provisionales o cuestiones inherentes es definitiva para efectos del amparo directo.</t>
+          <t>Las resoluciones dictadas durante la sustanciación del divorcio sin causa admiten recurso de revocación conforme a los arts. 685, 685 bis y 691 del CPC para CDMX.</t>
         </is>
       </c>
       <c r="R79" s="13" t="inlineStr">
         <is>
-          <t>Define vía de impugnación: amparo directo, no indirecto.</t>
+          <t>Vía expedita contra resoluciones intermedias en divorcio incausado CDMX.</t>
         </is>
       </c>
       <c r="S79" s="13" t="inlineStr">
         <is>
-          <t>Importante para no equivocarse de vía. Si tu sentencia incluye medidas sobre alimentos: amparo directo. Si solo es disolución limpia: dependerá del caso.</t>
+          <t>Antes era confusa la vía. Ahora con esta tesis se aplica revocación. Permite revisar rápidamente medidas provisionales sobre alimentos o convivencia.</t>
         </is>
       </c>
       <c r="T79" s="13" t="inlineStr"/>
       <c r="U79" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029853</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031170</t>
         </is>
       </c>
       <c r="V79" s="13" t="inlineStr">
         <is>
-          <t>divorcio incausado · amparo directo · alimentos</t>
+          <t>divorcio incausado · revocación · CDMX · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="80" ht="80" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>civ-ext-003</t>
+          <t>fam-div-002</t>
         </is>
       </c>
       <c r="B80" s="11" t="n">
@@ -11098,12 +11098,12 @@
       </c>
       <c r="E80" s="11" t="inlineStr">
         <is>
-          <t>Extinción de dominio</t>
+          <t>Divorcio sin expresión de causa</t>
         </is>
       </c>
       <c r="F80" s="11" t="inlineStr">
         <is>
-          <t>Comportarse como dueño — concepto</t>
+          <t>Amparo directo contra sentencia</t>
         </is>
       </c>
       <c r="G80" s="11" t="inlineStr">
@@ -11128,57 +11128,57 @@
       </c>
       <c r="K80" s="12" t="inlineStr">
         <is>
-          <t>ACCIÓN DE EXTINCIÓN DE DOMINIO. CONCEPTO DE "COMPORTARSE U OSTENTARSE COMO DUEÑO", PARA LOS EFECTOS DE LA LEY FEDERAL DE EXTINCIÓN DE DOMINIO (ABROGADA).</t>
+          <t>AMPARO DIRECTO. PROCEDE CONTRA LA SENTENCIA QUE DECLARA LA DISOLUCIÓN DEL VÍNCULO MATRIMONIAL EN UN JUICIO DE DIVORCIO SIN EXPRESIÓN DE CAUSA Y RESUELVE PROVISIONALMENTE SOBRE LOS ALIMENTOS U OTRAS CUESTIONES INHERENTES.</t>
         </is>
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>2024407</t>
+          <t>2029853</t>
         </is>
       </c>
       <c r="M80" s="11" t="inlineStr"/>
       <c r="N80" s="11" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2024-2025</t>
         </is>
       </c>
       <c r="O80" s="11" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P80" s="11" t="inlineStr"/>
       <c r="Q80" s="11" t="inlineStr">
         <is>
-          <t>El "comportarse u ostentarse como dueño" requiere acreditar actos materiales objetivos: posesión, administración, disposición, sin que baste la mera titularidad registral.</t>
+          <t>La sentencia de divorcio sin expresión de causa que resuelve sobre alimentos provisionales o cuestiones inherentes es definitiva para efectos del amparo directo.</t>
         </is>
       </c>
       <c r="R80" s="11" t="inlineStr">
         <is>
-          <t>Estándar para acreditar legitimación pasiva en extinción.</t>
+          <t>Define vía de impugnación: amparo directo, no indirecto.</t>
         </is>
       </c>
       <c r="S80" s="11" t="inlineStr">
         <is>
-          <t>Defensa: probar que tu cliente solo era titular registral, no se ostentaba como dueño.</t>
+          <t>Importante para no equivocarse de vía. Si tu sentencia incluye medidas sobre alimentos: amparo directo. Si solo es disolución limpia: dependerá del caso.</t>
         </is>
       </c>
       <c r="T80" s="11" t="inlineStr"/>
       <c r="U80" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024407</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029853</t>
         </is>
       </c>
       <c r="V80" s="11" t="inlineStr">
         <is>
-          <t>extinción dominio · ostentación · comportamiento · LFED</t>
+          <t>divorcio incausado · amparo directo · alimentos</t>
         </is>
       </c>
     </row>
     <row r="81" ht="80" customHeight="1">
       <c r="A81" s="13" t="inlineStr">
         <is>
-          <t>civ-fid-003</t>
+          <t>civ-ext-003</t>
         </is>
       </c>
       <c r="B81" s="13" t="n">
@@ -11196,12 +11196,12 @@
       </c>
       <c r="E81" s="13" t="inlineStr">
         <is>
-          <t>Fideicomisos</t>
+          <t>Extinción de dominio</t>
         </is>
       </c>
       <c r="F81" s="13" t="inlineStr">
         <is>
-          <t>Fideicomiso de garantía y mediación — avalúo</t>
+          <t>Comportarse como dueño — concepto</t>
         </is>
       </c>
       <c r="G81" s="13" t="inlineStr">
@@ -11226,18 +11226,18 @@
       </c>
       <c r="K81" s="14" t="inlineStr">
         <is>
-          <t>FIDEICOMISO EN GARANTÍA DERIVADO DE UN CONVENIO DE MEDIACIÓN. CUANDO SE PRETENDA SU EJECUCIÓN JUDICIAL DEBE EXHIBIRSE EL AVALÚO DEL BIEN INMUEBLE DADO EN GARANTÍA, AL SER UN ELEMENTO DE LA ACCIÓN CONFORME AL ARTÍCULO 1414 BIS DEL CÓDIGO DE COMERCIO.</t>
+          <t>ACCIÓN DE EXTINCIÓN DE DOMINIO. CONCEPTO DE "COMPORTARSE U OSTENTARSE COMO DUEÑO", PARA LOS EFECTOS DE LA LEY FEDERAL DE EXTINCIÓN DE DOMINIO (ABROGADA).</t>
         </is>
       </c>
       <c r="L81" s="13" t="inlineStr">
         <is>
-          <t>2027244</t>
+          <t>2024407</t>
         </is>
       </c>
       <c r="M81" s="13" t="inlineStr"/>
       <c r="N81" s="13" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="O81" s="13" t="inlineStr">
@@ -11248,35 +11248,35 @@
       <c r="P81" s="13" t="inlineStr"/>
       <c r="Q81" s="13" t="inlineStr">
         <is>
-          <t>Para ejecutar judicialmente fideicomiso de garantía constituido por convenio de mediación, el actor DEBE exhibir avalúo del bien al promover. Sin avalúo, la acción es improcedente.</t>
+          <t>El "comportarse u ostentarse como dueño" requiere acreditar actos materiales objetivos: posesión, administración, disposición, sin que baste la mera titularidad registral.</t>
         </is>
       </c>
       <c r="R81" s="13" t="inlineStr">
         <is>
-          <t>Requisito formal estricto para ejecutar fideicomiso de garantía vía mediación.</t>
+          <t>Estándar para acreditar legitimación pasiva en extinción.</t>
         </is>
       </c>
       <c r="S81" s="13" t="inlineStr">
         <is>
-          <t>Antes de demandar ejecución hay que conseguir avalúo de perito autorizado.</t>
+          <t>Defensa: probar que tu cliente solo era titular registral, no se ostentaba como dueño.</t>
         </is>
       </c>
       <c r="T81" s="13" t="inlineStr"/>
       <c r="U81" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027244</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024407</t>
         </is>
       </c>
       <c r="V81" s="13" t="inlineStr">
         <is>
-          <t>fideicomiso garantía · mediación · art. 1414 bis Cco · avalúo</t>
+          <t>extinción dominio · ostentación · comportamiento · LFED</t>
         </is>
       </c>
     </row>
     <row r="82" ht="80" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>auto-2032124</t>
+          <t>civ-fid-003</t>
         </is>
       </c>
       <c r="B82" s="11" t="n">
@@ -11294,12 +11294,12 @@
       </c>
       <c r="E82" s="11" t="inlineStr">
         <is>
-          <t>Juicio hipotecario</t>
+          <t>Fideicomisos</t>
         </is>
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>Actualización automática semanal</t>
+          <t>Fideicomiso de garantía y mediación — avalúo</t>
         </is>
       </c>
       <c r="G82" s="11" t="inlineStr">
@@ -11309,7 +11309,7 @@
       </c>
       <c r="H82" s="11" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I82" s="11" t="inlineStr">
@@ -11324,57 +11324,57 @@
       </c>
       <c r="K82" s="12" t="inlineStr">
         <is>
-          <t>CRÉDITOS HIPOTECARIOS OTORGADOS POR LAS INSTITUCIONES FINANCIERAS A SUS PERSONAS TRABAJADORAS. EL ESTUDIO SOBRE LA MODIFICACIÓN DE LAS CLÁUSULAS QUE CONTENGAN UN BENEFICIO OTORGADO DERIVADO DE LA RELACIÓN LABORAL PROCEDE EN ESTA VÍA.</t>
+          <t>FIDEICOMISO EN GARANTÍA DERIVADO DE UN CONVENIO DE MEDIACIÓN. CUANDO SE PRETENDA SU EJECUCIÓN JUDICIAL DEBE EXHIBIRSE EL AVALÚO DEL BIEN INMUEBLE DADO EN GARANTÍA, AL SER UN ELEMENTO DE LA ACCIÓN CONFORME AL ARTÍCULO 1414 BIS DEL CÓDIGO DE COMERCIO.</t>
         </is>
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>2032124</t>
+          <t>2027244</t>
         </is>
       </c>
       <c r="M82" s="11" t="inlineStr"/>
       <c r="N82" s="11" t="inlineStr">
         <is>
-          <t>viernes 15 de mayo de 2026 10:20 h</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="O82" s="11" t="inlineStr">
         <is>
-          <t>Semanario Judicial de la Federación — captura automática</t>
+          <t>Gaceta SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P82" s="11" t="inlineStr"/>
       <c r="Q82" s="11" t="inlineStr">
         <is>
-          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
+          <t>Para ejecutar judicialmente fideicomiso de garantía constituido por convenio de mediación, el actor DEBE exhibir avalúo del bien al promover. Sin avalúo, la acción es improcedente.</t>
         </is>
       </c>
       <c r="R82" s="11" t="inlineStr">
         <is>
-          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
+          <t>Requisito formal estricto para ejecutar fideicomiso de garantía vía mediación.</t>
         </is>
       </c>
       <c r="S82" s="11" t="inlineStr">
         <is>
-          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
+          <t>Antes de demandar ejecución hay que conseguir avalúo de perito autorizado.</t>
         </is>
       </c>
       <c r="T82" s="11" t="inlineStr"/>
       <c r="U82" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032124</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027244</t>
         </is>
       </c>
       <c r="V82" s="11" t="inlineStr">
         <is>
-          <t>Juicio hipotecario · actualización automática</t>
+          <t>fideicomiso garantía · mediación · art. 1414 bis Cco · avalúo</t>
         </is>
       </c>
     </row>
     <row r="83" ht="80" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>civ-hip-003</t>
+          <t>auto-2032124</t>
         </is>
       </c>
       <c r="B83" s="13" t="n">
@@ -11397,7 +11397,7 @@
       </c>
       <c r="F83" s="13" t="inlineStr">
         <is>
-          <t>Intereses y anatocismo</t>
+          <t>Actualización automática semanal</t>
         </is>
       </c>
       <c r="G83" s="13" t="inlineStr">
@@ -11407,7 +11407,7 @@
       </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I83" s="13" t="inlineStr">
@@ -11417,54 +11417,62 @@
       </c>
       <c r="J83" s="13" t="inlineStr">
         <is>
-          <t>Federal — colegiados</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K83" s="14" t="inlineStr">
         <is>
-          <t>INTERESES MORATORIOS EN MUTUO HIPOTECARIO. SU CAPITALIZACIÓN REQUIERE PACTO EXPRESO Y POSTERIOR A SU CAUSACIÓN.</t>
+          <t>CRÉDITOS HIPOTECARIOS OTORGADOS POR LAS INSTITUCIONES FINANCIERAS A SUS PERSONAS TRABAJADORAS. EL ESTUDIO SOBRE LA MODIFICACIÓN DE LAS CLÁUSULAS QUE CONTENGAN UN BENEFICIO OTORGADO DERIVADO DE LA RELACIÓN LABORAL PROCEDE EN ESTA VÍA.</t>
         </is>
       </c>
       <c r="L83" s="13" t="inlineStr">
         <is>
-          <t>200721</t>
+          <t>2032124</t>
         </is>
       </c>
       <c r="M83" s="13" t="inlineStr"/>
-      <c r="N83" s="13" t="inlineStr"/>
-      <c r="O83" s="13" t="inlineStr"/>
+      <c r="N83" s="13" t="inlineStr">
+        <is>
+          <t>viernes 15 de mayo de 2026 10:20 h</t>
+        </is>
+      </c>
+      <c r="O83" s="13" t="inlineStr">
+        <is>
+          <t>Semanario Judicial de la Federación — captura automática</t>
+        </is>
+      </c>
       <c r="P83" s="13" t="inlineStr"/>
       <c r="Q83" s="13" t="inlineStr">
         <is>
-          <t>La capitalización de intereses (anatocismo) en mutuo hipotecario civil solo es válida cuando se pacta por escrito y POSTERIORMENTE a que los intereses se causaron. Pactos previos genéricos de capitalización son nulos.</t>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
         </is>
       </c>
       <c r="R83" s="13" t="inlineStr">
         <is>
-          <t>Defensa estándar del deudor en hipotecarios de banca.</t>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
         </is>
       </c>
       <c r="S83" s="13" t="inlineStr">
         <is>
-          <t>El art. 2397 CCCDMX prohíbe el pacto anticipado de capitalización. En la práctica, las pólizas bancarias suelen incluir cláusula que se debe atacar como nula. Estudiar junto con criterios de Contradicción de Tesis 31/98 (anatocismo).</t>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
         </is>
       </c>
       <c r="T83" s="13" t="inlineStr"/>
       <c r="U83" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/164463</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032124</t>
         </is>
       </c>
       <c r="V83" s="13" t="inlineStr">
         <is>
-          <t>intereses · anatocismo · art. 2397 CCCDMX</t>
+          <t>Juicio hipotecario · actualización automática</t>
         </is>
       </c>
     </row>
     <row r="84" ht="80" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>civ-hip-004</t>
+          <t>civ-hip-003</t>
         </is>
       </c>
       <c r="B84" s="11" t="n">
@@ -11487,7 +11495,7 @@
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>Apelación en efecto devolutivo</t>
+          <t>Intereses y anatocismo</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
@@ -11497,7 +11505,7 @@
       </c>
       <c r="H84" s="11" t="inlineStr">
         <is>
-          <t>Novena Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I84" s="11" t="inlineStr">
@@ -11507,62 +11515,54 @@
       </c>
       <c r="J84" s="11" t="inlineStr">
         <is>
-          <t>CDMX</t>
+          <t>Federal — colegiados</t>
         </is>
       </c>
       <c r="K84" s="12" t="inlineStr">
         <is>
-          <t>JUICIO ESPECIAL HIPOTECARIO, APELACIÓN EN EL. DEBE ADMITIRSE EN EL EFECTO DEVOLUTIVO CONFORME AL ARTÍCULO 714 DEL CÓDIGO DE PROCEDIMIENTOS CIVILES PARA EL DISTRITO FEDERAL.</t>
+          <t>INTERESES MORATORIOS EN MUTUO HIPOTECARIO. SU CAPITALIZACIÓN REQUIERE PACTO EXPRESO Y POSTERIOR A SU CAUSACIÓN.</t>
         </is>
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>162554</t>
+          <t>200721</t>
         </is>
       </c>
       <c r="M84" s="11" t="inlineStr"/>
-      <c r="N84" s="11" t="inlineStr">
-        <is>
-          <t>Novena Época</t>
-        </is>
-      </c>
-      <c r="O84" s="11" t="inlineStr">
-        <is>
-          <t>Semanario Judicial de la Federación — VERIFICADO</t>
-        </is>
-      </c>
+      <c r="N84" s="11" t="inlineStr"/>
+      <c r="O84" s="11" t="inlineStr"/>
       <c r="P84" s="11" t="inlineStr"/>
       <c r="Q84" s="11" t="inlineStr">
         <is>
-          <t>Las apelaciones interlocutorias en el juicio especial hipotecario CDMX se admiten en efecto devolutivo, sin suspender la ejecución, conforme al art. 714 CPCDMX.</t>
+          <t>La capitalización de intereses (anatocismo) en mutuo hipotecario civil solo es válida cuando se pacta por escrito y POSTERIORMENTE a que los intereses se causaron. Pactos previos genéricos de capitalización son nulos.</t>
         </is>
       </c>
       <c r="R84" s="11" t="inlineStr">
         <is>
-          <t>Acreedor mantiene ejecución pese a apelaciones del deudor.</t>
+          <t>Defensa estándar del deudor en hipotecarios de banca.</t>
         </is>
       </c>
       <c r="S84" s="11" t="inlineStr">
         <is>
-          <t>Defensa del banco/acreedor: las apelaciones no detienen el remate. El deudor debe ir por amparo indirecto si quiere suspender.</t>
+          <t>El art. 2397 CCCDMX prohíbe el pacto anticipado de capitalización. En la práctica, las pólizas bancarias suelen incluir cláusula que se debe atacar como nula. Estudiar junto con criterios de Contradicción de Tesis 31/98 (anatocismo).</t>
         </is>
       </c>
       <c r="T84" s="11" t="inlineStr"/>
       <c r="U84" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/162554</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/164463</t>
         </is>
       </c>
       <c r="V84" s="11" t="inlineStr">
         <is>
-          <t>hipotecario · apelación · art. 714 CPCDMX · efecto devolutivo</t>
+          <t>intereses · anatocismo · art. 2397 CCCDMX</t>
         </is>
       </c>
     </row>
     <row r="85" ht="80" customHeight="1">
       <c r="A85" s="13" t="inlineStr">
         <is>
-          <t>civ-hip-005</t>
+          <t>civ-hip-004</t>
         </is>
       </c>
       <c r="B85" s="13" t="n">
@@ -11585,7 +11585,7 @@
       </c>
       <c r="F85" s="13" t="inlineStr">
         <is>
-          <t>Ejecución limitada al bien hipotecado</t>
+          <t>Apelación en efecto devolutivo</t>
         </is>
       </c>
       <c r="G85" s="13" t="inlineStr">
@@ -11605,17 +11605,17 @@
       </c>
       <c r="J85" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>CDMX</t>
         </is>
       </c>
       <c r="K85" s="14" t="inlineStr">
         <is>
-          <t>JUICIO HIPOTECARIO. ES JURÍDICAMENTE IMPOSIBLE DESPACHAR EJECUCIÓN EN UN INMUEBLE DISTINTO DEL BIEN MATERIA DE LA CONDENA.</t>
+          <t>JUICIO ESPECIAL HIPOTECARIO, APELACIÓN EN EL. DEBE ADMITIRSE EN EL EFECTO DEVOLUTIVO CONFORME AL ARTÍCULO 714 DEL CÓDIGO DE PROCEDIMIENTOS CIVILES PARA EL DISTRITO FEDERAL.</t>
         </is>
       </c>
       <c r="L85" s="13" t="inlineStr">
         <is>
-          <t>180865</t>
+          <t>162554</t>
         </is>
       </c>
       <c r="M85" s="13" t="inlineStr"/>
@@ -11626,41 +11626,41 @@
       </c>
       <c r="O85" s="13" t="inlineStr">
         <is>
-          <t>SJF — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — VERIFICADO</t>
         </is>
       </c>
       <c r="P85" s="13" t="inlineStr"/>
       <c r="Q85" s="13" t="inlineStr">
         <is>
-          <t>La acción real hipotecaria solo permite ejecutar sobre el bien hipotecado. No puede ampliarse a otros bienes del deudor mediante convenios anteriores a la sentencia.</t>
+          <t>Las apelaciones interlocutorias en el juicio especial hipotecario CDMX se admiten en efecto devolutivo, sin suspender la ejecución, conforme al art. 714 CPCDMX.</t>
         </is>
       </c>
       <c r="R85" s="13" t="inlineStr">
         <is>
-          <t>Límite de garantía real del juicio hipotecario.</t>
+          <t>Acreedor mantiene ejecución pese a apelaciones del deudor.</t>
         </is>
       </c>
       <c r="S85" s="13" t="inlineStr">
         <is>
-          <t>El acreedor que quiera ir contra otros bienes debe abrir vía ordinaria adicional. Defensa del deudor: oponer la limitación si el ejecutor intenta otros inmuebles.</t>
+          <t>Defensa del banco/acreedor: las apelaciones no detienen el remate. El deudor debe ir por amparo indirecto si quiere suspender.</t>
         </is>
       </c>
       <c r="T85" s="13" t="inlineStr"/>
       <c r="U85" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/180865</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/162554</t>
         </is>
       </c>
       <c r="V85" s="13" t="inlineStr">
         <is>
-          <t>hipotecario · acción real · ejecución limitada</t>
+          <t>hipotecario · apelación · art. 714 CPCDMX · efecto devolutivo</t>
         </is>
       </c>
     </row>
     <row r="86" ht="80" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>sen-019</t>
+          <t>civ-hip-005</t>
         </is>
       </c>
       <c r="B86" s="11" t="n">
@@ -11678,22 +11678,22 @@
       </c>
       <c r="E86" s="11" t="inlineStr">
         <is>
-          <t>Notificaciones — domicilio convencional vs. real</t>
+          <t>Juicio hipotecario</t>
         </is>
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>Línea de Colegiados Primer Circuito (CDMX)</t>
+          <t>Ejecución limitada al bien hipotecado</t>
         </is>
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>sentencia hito</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H86" s="11" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Novena Época</t>
         </is>
       </c>
       <c r="I86" s="11" t="inlineStr">
@@ -11703,58 +11703,62 @@
       </c>
       <c r="J86" s="11" t="inlineStr">
         <is>
-          <t>Primer Circuito — CDMX</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K86" s="12" t="inlineStr">
         <is>
-          <t>Notificación personal — preeminencia del domicilio real cuando consta en autos</t>
+          <t>JUICIO HIPOTECARIO. ES JURÍDICAMENTE IMPOSIBLE DESPACHAR EJECUCIÓN EN UN INMUEBLE DISTINTO DEL BIEN MATERIA DE LA CONDENA.</t>
         </is>
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>Tesis del Primer Circuito — múltiples colegiados civiles</t>
+          <t>180865</t>
         </is>
       </c>
       <c r="M86" s="11" t="inlineStr"/>
       <c r="N86" s="11" t="inlineStr">
         <is>
-          <t>Línea consolidada</t>
-        </is>
-      </c>
-      <c r="O86" s="11" t="inlineStr"/>
+          <t>Novena Época</t>
+        </is>
+      </c>
+      <c r="O86" s="11" t="inlineStr">
+        <is>
+          <t>SJF — VERIFICADO</t>
+        </is>
+      </c>
       <c r="P86" s="11" t="inlineStr"/>
       <c r="Q86" s="11" t="inlineStr">
         <is>
-          <t>Aunque exista domicilio convencional pactado, si en autos consta el domicilio real del demandado y el convencional resulta inhábil, el actuario debe notificar en el real para garantizar emplazamiento efectivo y derecho de audiencia.</t>
+          <t>La acción real hipotecaria solo permite ejecutar sobre el bien hipotecado. No puede ampliarse a otros bienes del deudor mediante convenios anteriores a la sentencia.</t>
         </is>
       </c>
       <c r="R86" s="11" t="inlineStr">
         <is>
-          <t>Defensa nuclear contra emplazamientos ficticios.</t>
+          <t>Límite de garantía real del juicio hipotecario.</t>
         </is>
       </c>
       <c r="S86" s="11" t="inlineStr">
         <is>
-          <t>En juicios ejecutivos y especiales hipotecarios, el demandado que no fue notificado personalmente y no tuvo oportunidad real de defensa puede pedir nulidad del emplazamiento. Ofrecer pruebas del domicilio real anteriores al juicio.</t>
+          <t>El acreedor que quiera ir contra otros bienes debe abrir vía ordinaria adicional. Defensa del deudor: oponer la limitación si el ejecutor intenta otros inmuebles.</t>
         </is>
       </c>
       <c r="T86" s="11" t="inlineStr"/>
       <c r="U86" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2030925</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/180865</t>
         </is>
       </c>
       <c r="V86" s="11" t="inlineStr">
         <is>
-          <t>notificación · emplazamiento · domicilio real · Primer Circuito</t>
+          <t>hipotecario · acción real · ejecución limitada</t>
         </is>
       </c>
     </row>
     <row r="87" ht="80" customHeight="1">
       <c r="A87" s="13" t="inlineStr">
         <is>
-          <t>fam-com-001</t>
+          <t>sen-019</t>
         </is>
       </c>
       <c r="B87" s="13" t="n">
@@ -11772,22 +11776,22 @@
       </c>
       <c r="E87" s="13" t="inlineStr">
         <is>
-          <t>Pensión compensatoria</t>
+          <t>Notificaciones — domicilio convencional vs. real</t>
         </is>
       </c>
       <c r="F87" s="13" t="inlineStr">
         <is>
-          <t>Inversión de carga probatoria</t>
+          <t>Línea de Colegiados Primer Circuito (CDMX)</t>
         </is>
       </c>
       <c r="G87" s="13" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>sentencia hito</t>
         </is>
       </c>
       <c r="H87" s="13" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I87" s="13" t="inlineStr">
@@ -11797,62 +11801,58 @@
       </c>
       <c r="J87" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Primer Circuito — CDMX</t>
         </is>
       </c>
       <c r="K87" s="14" t="inlineStr">
         <is>
-          <t>INVERSIÓN DE LA CARGA DE LA PRUEBA EN MATERIA FAMILIAR. CUANDO SE DEMANDA UNA PENSIÓN COMPENSATORIA Y SE PRODUCE AQUÉLLA, LA PERSONA JUZGADORA TIENE EL DEBER DE HACERLO SABER EXPRESA Y OPORTUNAMENTE A LA PARTE SOBRE LA QUE RECAE.</t>
+          <t>Notificación personal — preeminencia del domicilio real cuando consta en autos</t>
         </is>
       </c>
       <c r="L87" s="13" t="inlineStr">
         <is>
-          <t>2031387</t>
+          <t>Tesis del Primer Circuito — múltiples colegiados civiles</t>
         </is>
       </c>
       <c r="M87" s="13" t="inlineStr"/>
       <c r="N87" s="13" t="inlineStr">
         <is>
-          <t>2025-2026</t>
-        </is>
-      </c>
-      <c r="O87" s="13" t="inlineStr">
-        <is>
-          <t>SJF — VERIFICADO</t>
-        </is>
-      </c>
+          <t>Línea consolidada</t>
+        </is>
+      </c>
+      <c r="O87" s="13" t="inlineStr"/>
       <c r="P87" s="13" t="inlineStr"/>
       <c r="Q87" s="13" t="inlineStr">
         <is>
-          <t>En juicios de pensión compensatoria, cuando opera la inversión de carga probatoria, el juez tiene deber DE OFICIO de notificar formalmente a la parte sobre la que recae para garantizar defensa adecuada.</t>
+          <t>Aunque exista domicilio convencional pactado, si en autos consta el domicilio real del demandado y el convencional resulta inhábil, el actuario debe notificar en el real para garantizar emplazamiento efectivo y derecho de audiencia.</t>
         </is>
       </c>
       <c r="R87" s="13" t="inlineStr">
         <is>
-          <t>Garantía procesal en juicios de compensación / pensión.</t>
+          <t>Defensa nuclear contra emplazamientos ficticios.</t>
         </is>
       </c>
       <c r="S87" s="13" t="inlineStr">
         <is>
-          <t>Defensa del deudor alimentario: si no le informaron expresamente la inversión, puede pedir nulidad de actuaciones. Defensa del acreedor: solicitar al juez que haga la notificación formal.</t>
+          <t>En juicios ejecutivos y especiales hipotecarios, el demandado que no fue notificado personalmente y no tuvo oportunidad real de defensa puede pedir nulidad del emplazamiento. Ofrecer pruebas del domicilio real anteriores al juicio.</t>
         </is>
       </c>
       <c r="T87" s="13" t="inlineStr"/>
       <c r="U87" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031387</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2030925</t>
         </is>
       </c>
       <c r="V87" s="13" t="inlineStr">
         <is>
-          <t>pensión compensatoria · carga probatoria · 12a Época</t>
+          <t>notificación · emplazamiento · domicilio real · Primer Circuito</t>
         </is>
       </c>
     </row>
     <row r="88" ht="80" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>civ-usu-003</t>
+          <t>fam-com-001</t>
         </is>
       </c>
       <c r="B88" s="11" t="n">
@@ -11870,22 +11870,22 @@
       </c>
       <c r="E88" s="11" t="inlineStr">
         <is>
-          <t>Usucapión / Prescripción positiva</t>
+          <t>Pensión compensatoria</t>
         </is>
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>Pericial topográfica / agrimensura</t>
+          <t>Inversión de carga probatoria</t>
         </is>
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>jurisprudencia</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H88" s="11" t="inlineStr">
         <is>
-          <t>Novena Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
@@ -11895,58 +11895,62 @@
       </c>
       <c r="J88" s="11" t="inlineStr">
         <is>
-          <t>Federal — colegiados</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr">
         <is>
-          <t>PERICIAL EN AGRIMENSURA. ES IDÓNEA PARA DEMOSTRAR LA IDENTIDAD DEL PREDIO MATERIA DE LA USUCAPIÓN, CUANDO ESTE NO APARECE INDIVIDUALIZADO EN EL REGISTRO PÚBLICO DE LA PROPIEDAD.</t>
+          <t>INVERSIÓN DE LA CARGA DE LA PRUEBA EN MATERIA FAMILIAR. CUANDO SE DEMANDA UNA PENSIÓN COMPENSATORIA Y SE PRODUCE AQUÉLLA, LA PERSONA JUZGADORA TIENE EL DEBER DE HACERLO SABER EXPRESA Y OPORTUNAMENTE A LA PARTE SOBRE LA QUE RECAE.</t>
         </is>
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>190377</t>
+          <t>2031387</t>
         </is>
       </c>
       <c r="M88" s="11" t="inlineStr"/>
-      <c r="N88" s="11" t="inlineStr"/>
+      <c r="N88" s="11" t="inlineStr">
+        <is>
+          <t>2025-2026</t>
+        </is>
+      </c>
       <c r="O88" s="11" t="inlineStr">
         <is>
-          <t>SJF y su Gaceta, Novena Época — VERIFICADO en SJF2</t>
+          <t>SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P88" s="11" t="inlineStr"/>
       <c r="Q88" s="11" t="inlineStr">
         <is>
-          <t>Cuando el inmueble se desprende de una superficie mayor o no aparece individualizado registralmente, la pericial topográfica es la prueba idónea para acreditar la identidad y localización exacta del predio que se pretende prescribir.</t>
+          <t>En juicios de pensión compensatoria, cuando opera la inversión de carga probatoria, el juez tiene deber DE OFICIO de notificar formalmente a la parte sobre la que recae para garantizar defensa adecuada.</t>
         </is>
       </c>
       <c r="R88" s="11" t="inlineStr">
         <is>
-          <t>Indispensable en cualquier predio desprendido de matriz mayor.</t>
+          <t>Garantía procesal en juicios de compensación / pensión.</t>
         </is>
       </c>
       <c r="S88" s="11" t="inlineStr">
         <is>
-          <t>Sin pericial topográfica el juicio se expone a falta de identidad del bien. Hay que ofrecerla desde la demanda con cuestionario que incluya: medidas, colindancias, superficie y ubicación cartográfica.</t>
+          <t>Defensa del deudor alimentario: si no le informaron expresamente la inversión, puede pedir nulidad de actuaciones. Defensa del acreedor: solicitar al juez que haga la notificación formal.</t>
         </is>
       </c>
       <c r="T88" s="11" t="inlineStr"/>
       <c r="U88" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/190377</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031387</t>
         </is>
       </c>
       <c r="V88" s="11" t="inlineStr">
         <is>
-          <t>pericial · topografía · identidad del bien</t>
+          <t>pensión compensatoria · carga probatoria · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="89" ht="80" customHeight="1">
       <c r="A89" s="13" t="inlineStr">
         <is>
-          <t>civ-usu-005</t>
+          <t>civ-usu-003</t>
         </is>
       </c>
       <c r="B89" s="13" t="n">
@@ -11969,7 +11973,7 @@
       </c>
       <c r="F89" s="13" t="inlineStr">
         <is>
-          <t>Posesión derivada vs. originaria</t>
+          <t>Pericial topográfica / agrimensura</t>
         </is>
       </c>
       <c r="G89" s="13" t="inlineStr">
@@ -11979,7 +11983,7 @@
       </c>
       <c r="H89" s="13" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Novena Época</t>
         </is>
       </c>
       <c r="I89" s="13" t="inlineStr">
@@ -11989,54 +11993,58 @@
       </c>
       <c r="J89" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Federal — colegiados</t>
         </is>
       </c>
       <c r="K89" s="14" t="inlineStr">
         <is>
-          <t>POSESIÓN DERIVADA. NO PRODUCE LOS EFECTOS DE LA POSESIÓN ORIGINARIA PARA EFECTOS DE LA PRESCRIPCIÓN ADQUISITIVA.</t>
+          <t>PERICIAL EN AGRIMENSURA. ES IDÓNEA PARA DEMOSTRAR LA IDENTIDAD DEL PREDIO MATERIA DE LA USUCAPIÓN, CUANDO ESTE NO APARECE INDIVIDUALIZADO EN EL REGISTRO PÚBLICO DE LA PROPIEDAD.</t>
         </is>
       </c>
       <c r="L89" s="13" t="inlineStr">
         <is>
-          <t>2030499</t>
+          <t>190377</t>
         </is>
       </c>
       <c r="M89" s="13" t="inlineStr"/>
       <c r="N89" s="13" t="inlineStr"/>
-      <c r="O89" s="13" t="inlineStr"/>
+      <c r="O89" s="13" t="inlineStr">
+        <is>
+          <t>SJF y su Gaceta, Novena Época — VERIFICADO en SJF2</t>
+        </is>
+      </c>
       <c r="P89" s="13" t="inlineStr"/>
       <c r="Q89" s="13" t="inlineStr">
         <is>
-          <t>Quien posee por virtud de un título que reconoce dominio ajeno (arrendatario, comodatario, usufructuario, depositario) no posee en concepto de propietario y no puede usucapir, salvo intervertio possessionis acreditada.</t>
+          <t>Cuando el inmueble se desprende de una superficie mayor o no aparece individualizado registralmente, la pericial topográfica es la prueba idónea para acreditar la identidad y localización exacta del predio que se pretende prescribir.</t>
         </is>
       </c>
       <c r="R89" s="13" t="inlineStr">
         <is>
-          <t>Filtra acciones de usucapión espurias por arrendatarios o detentadores.</t>
+          <t>Indispensable en cualquier predio desprendido de matriz mayor.</t>
         </is>
       </c>
       <c r="S89" s="13" t="inlineStr">
         <is>
-          <t>El demandado por arrendamiento puede oponer la usucapión solo si demuestra que cambió el concepto de su posesión a originaria — hecho que rara vez se prueba.</t>
+          <t>Sin pericial topográfica el juicio se expone a falta de identidad del bien. Hay que ofrecerla desde la demanda con cuestionario que incluya: medidas, colindancias, superficie y ubicación cartográfica.</t>
         </is>
       </c>
       <c r="T89" s="13" t="inlineStr"/>
       <c r="U89" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2030499</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/190377</t>
         </is>
       </c>
       <c r="V89" s="13" t="inlineStr">
         <is>
-          <t>posesión derivada · concepto de propietario · interversión</t>
+          <t>pericial · topografía · identidad del bien</t>
         </is>
       </c>
     </row>
     <row r="90" ht="80" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>con-asa-001</t>
+          <t>civ-usu-005</t>
         </is>
       </c>
       <c r="B90" s="11" t="n">
@@ -12049,22 +12057,22 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>Civil — Condominio</t>
+          <t>Civil</t>
         </is>
       </c>
       <c r="E90" s="11" t="inlineStr">
         <is>
-          <t>Régimen de propiedad en condominio</t>
+          <t>Usucapión / Prescripción positiva</t>
         </is>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>Asambleas — convocatoria y validez</t>
+          <t>Posesión derivada vs. originaria</t>
         </is>
       </c>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>jurisprudencia</t>
         </is>
       </c>
       <c r="H90" s="11" t="inlineStr">
@@ -12079,17 +12087,17 @@
       </c>
       <c r="J90" s="11" t="inlineStr">
         <is>
-          <t>Federal — interpreta LPCI CDMX</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr">
         <is>
-          <t>ASAMBLEAS CONDOMINALES. LA INDEBIDA CONVOCATORIA AFECTA LA VALIDEZ DE LOS ACUERDOS Y PERMITE SU IMPUGNACIÓN.</t>
+          <t>POSESIÓN DERIVADA. NO PRODUCE LOS EFECTOS DE LA POSESIÓN ORIGINARIA PARA EFECTOS DE LA PRESCRIPCIÓN ADQUISITIVA.</t>
         </is>
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>Art. 32 LPCI CDMX</t>
+          <t>2030499</t>
         </is>
       </c>
       <c r="M90" s="11" t="inlineStr"/>
@@ -12098,35 +12106,35 @@
       <c r="P90" s="11" t="inlineStr"/>
       <c r="Q90" s="11" t="inlineStr">
         <is>
-          <t>La convocatoria debe respetar plazo, forma y orden del día (art. 32 LPCI CDMX). Su incumplimiento es causal de nulidad de los acuerdos adoptados, salvo ratificación expresa en asamblea posterior debidamente convocada.</t>
+          <t>Quien posee por virtud de un título que reconoce dominio ajeno (arrendatario, comodatario, usufructuario, depositario) no posee en concepto de propietario y no puede usucapir, salvo intervertio possessionis acreditada.</t>
         </is>
       </c>
       <c r="R90" s="11" t="inlineStr">
         <is>
-          <t>Defensa frecuente de minorías condominales.</t>
+          <t>Filtra acciones de usucapión espurias por arrendatarios o detentadores.</t>
         </is>
       </c>
       <c r="S90" s="11" t="inlineStr">
         <is>
-          <t>Conserva pruebas de cómo se realizó la convocatoria (carteles, mensajes, fotos). Plazo de impugnación es corto (60 días naturales en CDMX desde celebración o conocimiento).</t>
+          <t>El demandado por arrendamiento puede oponer la usucapión solo si demuestra que cambió el concepto de su posesión a originaria — hecho que rara vez se prueba.</t>
         </is>
       </c>
       <c r="T90" s="11" t="inlineStr"/>
       <c r="U90" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2028919</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2030499</t>
         </is>
       </c>
       <c r="V90" s="11" t="inlineStr">
         <is>
-          <t>asamblea · convocatoria · nulidad · LPCI CDMX</t>
+          <t>posesión derivada · concepto de propietario · interversión</t>
         </is>
       </c>
     </row>
     <row r="91" ht="80" customHeight="1">
       <c r="A91" s="13" t="inlineStr">
         <is>
-          <t>amp-cui-001</t>
+          <t>con-asa-001</t>
         </is>
       </c>
       <c r="B91" s="13" t="n">
@@ -12139,17 +12147,17 @@
       </c>
       <c r="D91" s="13" t="inlineStr">
         <is>
-          <t>Constitucional / DDHH</t>
+          <t>Civil — Condominio</t>
         </is>
       </c>
       <c r="E91" s="13" t="inlineStr">
         <is>
-          <t>Derecho humano al cuidado</t>
+          <t>Régimen de propiedad en condominio</t>
         </is>
       </c>
       <c r="F91" s="13" t="inlineStr">
         <is>
-          <t>Reconocimiento e interés legítimo</t>
+          <t>Asambleas — convocatoria y validez</t>
         </is>
       </c>
       <c r="G91" s="13" t="inlineStr">
@@ -12159,7 +12167,7 @@
       </c>
       <c r="H91" s="13" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I91" s="13" t="inlineStr">
@@ -12169,62 +12177,54 @@
       </c>
       <c r="J91" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Federal — interpreta LPCI CDMX</t>
         </is>
       </c>
       <c r="K91" s="14" t="inlineStr">
         <is>
-          <t>DERECHO HUMANO AL CUIDADO. IMPONE OBLIGACIONES DE CUYO CUMPLIMIENTO DEPENDE DIRECTAMENTE EL BIENESTAR DE LAS PERSONAS E INDIRECTAMENTE, POR INTERDEPENDENCIA, EL EJERCICIO EFECTIVO DE OTROS DERECHOS HUMANOS.</t>
+          <t>ASAMBLEAS CONDOMINALES. LA INDEBIDA CONVOCATORIA AFECTA LA VALIDEZ DE LOS ACUERDOS Y PERMITE SU IMPUGNACIÓN.</t>
         </is>
       </c>
       <c r="L91" s="13" t="inlineStr">
         <is>
-          <t>2032085</t>
+          <t>Art. 32 LPCI CDMX</t>
         </is>
       </c>
       <c r="M91" s="13" t="inlineStr"/>
-      <c r="N91" s="13" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="O91" s="13" t="inlineStr">
-        <is>
-          <t>SJF 12a Época — VERIFICADO</t>
-        </is>
-      </c>
+      <c r="N91" s="13" t="inlineStr"/>
+      <c r="O91" s="13" t="inlineStr"/>
       <c r="P91" s="13" t="inlineStr"/>
       <c r="Q91" s="13" t="inlineStr">
         <is>
-          <t>El cuidado se reconoce como derecho humano autónomo. El Estado tiene obligación de garantizarlo mediante políticas públicas, infraestructura social y reconocimiento del trabajo de cuidado no remunerado.</t>
+          <t>La convocatoria debe respetar plazo, forma y orden del día (art. 32 LPCI CDMX). Su incumplimiento es causal de nulidad de los acuerdos adoptados, salvo ratificación expresa en asamblea posterior debidamente convocada.</t>
         </is>
       </c>
       <c r="R91" s="13" t="inlineStr">
         <is>
-          <t>Pieza inaugural de un nuevo derecho humano en México.</t>
+          <t>Defensa frecuente de minorías condominales.</t>
         </is>
       </c>
       <c r="S91" s="13" t="inlineStr">
         <is>
-          <t>Marco para litigios sobre obligaciones del Estado en guarderías, cuidado de personas mayores, discapacidad y omisiones legislativas absolutas.</t>
+          <t>Conserva pruebas de cómo se realizó la convocatoria (carteles, mensajes, fotos). Plazo de impugnación es corto (60 días naturales en CDMX desde celebración o conocimiento).</t>
         </is>
       </c>
       <c r="T91" s="13" t="inlineStr"/>
       <c r="U91" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032085</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2028919</t>
         </is>
       </c>
       <c r="V91" s="13" t="inlineStr">
         <is>
-          <t>derecho al cuidado · 12a Época · DDHH · cuidadoras</t>
+          <t>asamblea · convocatoria · nulidad · LPCI CDMX</t>
         </is>
       </c>
     </row>
     <row r="92" ht="80" customHeight="1">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>amp-cui-002</t>
+          <t>amp-cui-001</t>
         </is>
       </c>
       <c r="B92" s="11" t="n">
@@ -12247,7 +12247,7 @@
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>Interés legítimo para combatir omisiones legislativas</t>
+          <t>Reconocimiento e interés legítimo</t>
         </is>
       </c>
       <c r="G92" s="11" t="inlineStr">
@@ -12272,12 +12272,12 @@
       </c>
       <c r="K92" s="12" t="inlineStr">
         <is>
-          <t>DERECHO HUMANO AL CUIDADO. LAS MUJERES QUE REALIZAN CUIDADOS SIMPLES O COTIDIANOS NO REMUNERADOS TIENEN INTERÉS LEGÍTIMO PARA RECLAMAR OMISIONES LEGISLATIVAS ABSOLUTAS QUE IMPIDAN SU PLENO EJERCICIO.</t>
+          <t>DERECHO HUMANO AL CUIDADO. IMPONE OBLIGACIONES DE CUYO CUMPLIMIENTO DEPENDE DIRECTAMENTE EL BIENESTAR DE LAS PERSONAS E INDIRECTAMENTE, POR INTERDEPENDENCIA, EL EJERCICIO EFECTIVO DE OTROS DERECHOS HUMANOS.</t>
         </is>
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>2032086</t>
+          <t>2032085</t>
         </is>
       </c>
       <c r="M92" s="11" t="inlineStr"/>
@@ -12294,35 +12294,35 @@
       <c r="P92" s="11" t="inlineStr"/>
       <c r="Q92" s="11" t="inlineStr">
         <is>
-          <t>Las mujeres que realizan trabajo de cuidados no remunerados tienen interés legítimo, sin necesidad de afectación individualizada estricta, para promover amparo contra omisiones legislativas absolutas en la materia.</t>
+          <t>El cuidado se reconoce como derecho humano autónomo. El Estado tiene obligación de garantizarlo mediante políticas públicas, infraestructura social y reconocimiento del trabajo de cuidado no remunerado.</t>
         </is>
       </c>
       <c r="R92" s="11" t="inlineStr">
         <is>
-          <t>Abre vía de amparo colectivo a millones de cuidadoras.</t>
+          <t>Pieza inaugural de un nuevo derecho humano en México.</t>
         </is>
       </c>
       <c r="S92" s="11" t="inlineStr">
         <is>
-          <t>Estrategia colectiva: amparos contra ausencia de legislación de cuidados. Beneficia particularmente a mujeres de bajos ingresos que sostienen familia.</t>
+          <t>Marco para litigios sobre obligaciones del Estado en guarderías, cuidado de personas mayores, discapacidad y omisiones legislativas absolutas.</t>
         </is>
       </c>
       <c r="T92" s="11" t="inlineStr"/>
       <c r="U92" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032086</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032085</t>
         </is>
       </c>
       <c r="V92" s="11" t="inlineStr">
         <is>
-          <t>cuidado · interés legítimo · omisión legislativa · perspectiva género</t>
+          <t>derecho al cuidado · 12a Época · DDHH · cuidadoras</t>
         </is>
       </c>
     </row>
     <row r="93" ht="80" customHeight="1">
       <c r="A93" s="13" t="inlineStr">
         <is>
-          <t>amp-gen-001</t>
+          <t>amp-cui-002</t>
         </is>
       </c>
       <c r="B93" s="13" t="n">
@@ -12340,12 +12340,12 @@
       </c>
       <c r="E93" s="13" t="inlineStr">
         <is>
-          <t>Perspectiva de género interseccional</t>
+          <t>Derecho humano al cuidado</t>
         </is>
       </c>
       <c r="F93" s="13" t="inlineStr">
         <is>
-          <t>Acceso a la justicia para mujeres cuidadoras</t>
+          <t>Interés legítimo para combatir omisiones legislativas</t>
         </is>
       </c>
       <c r="G93" s="13" t="inlineStr">
@@ -12370,12 +12370,12 @@
       </c>
       <c r="K93" s="14" t="inlineStr">
         <is>
-          <t>ACCESO A LA JUSTICIA EN CONDICIONES DE IGUALDAD SUSTANTIVA. LAS MANIFESTACIONES DE MUJERES QUE AFIRMAN REALIZAR LABORES DE CUIDADO NO REMUNERADAS DEBEN VALORARSE CON PERSPECTIVA DE GÉNERO INTERSECCIONAL.</t>
+          <t>DERECHO HUMANO AL CUIDADO. LAS MUJERES QUE REALIZAN CUIDADOS SIMPLES O COTIDIANOS NO REMUNERADOS TIENEN INTERÉS LEGÍTIMO PARA RECLAMAR OMISIONES LEGISLATIVAS ABSOLUTAS QUE IMPIDAN SU PLENO EJERCICIO.</t>
         </is>
       </c>
       <c r="L93" s="13" t="inlineStr">
         <is>
-          <t>2032067</t>
+          <t>2032086</t>
         </is>
       </c>
       <c r="M93" s="13" t="inlineStr"/>
@@ -12392,35 +12392,35 @@
       <c r="P93" s="13" t="inlineStr"/>
       <c r="Q93" s="13" t="inlineStr">
         <is>
-          <t>En procesos donde las mujeres afirman dedicarse a labores de cuidado, sus manifestaciones deben valorarse con perspectiva de género interseccional (considerando clase, edad, etnia, discapacidad y otros factores).</t>
+          <t>Las mujeres que realizan trabajo de cuidados no remunerados tienen interés legítimo, sin necesidad de afectación individualizada estricta, para promover amparo contra omisiones legislativas absolutas en la materia.</t>
         </is>
       </c>
       <c r="R93" s="13" t="inlineStr">
         <is>
-          <t>Estándar probatorio favorable para mujeres en juicios civiles, familiares, laborales.</t>
+          <t>Abre vía de amparo colectivo a millones de cuidadoras.</t>
         </is>
       </c>
       <c r="S93" s="13" t="inlineStr">
         <is>
-          <t>En alimentos, pensiones, compensación por trabajo doméstico y otros litigios, el juez debe creer y valorar con flexibilidad las declaraciones de mujeres cuidadoras.</t>
+          <t>Estrategia colectiva: amparos contra ausencia de legislación de cuidados. Beneficia particularmente a mujeres de bajos ingresos que sostienen familia.</t>
         </is>
       </c>
       <c r="T93" s="13" t="inlineStr"/>
       <c r="U93" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032067</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032086</t>
         </is>
       </c>
       <c r="V93" s="13" t="inlineStr">
         <is>
-          <t>perspectiva género · interseccional · acceso justicia · 12a Época</t>
+          <t>cuidado · interés legítimo · omisión legislativa · perspectiva género</t>
         </is>
       </c>
     </row>
     <row r="94" ht="80" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>fis-cfd-002</t>
+          <t>auto-2032154</t>
         </is>
       </c>
       <c r="B94" s="11" t="n">
@@ -12433,22 +12433,22 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>Fiscal</t>
+          <t>Constitucional / DDHH</t>
         </is>
       </c>
       <c r="E94" s="11" t="inlineStr">
         <is>
-          <t>Comprobantes fiscales (CFDI)</t>
+          <t>Perspectiva de género</t>
         </is>
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>69-B — recurso de revocación y buzón tributario</t>
+          <t>Actualización automática semanal</t>
         </is>
       </c>
       <c r="G94" s="11" t="inlineStr">
         <is>
-          <t>jurisprudencia</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H94" s="11" t="inlineStr">
@@ -12468,57 +12468,57 @@
       </c>
       <c r="K94" s="12" t="inlineStr">
         <is>
-          <t>RECURSO DE REVOCACIÓN CONTRA LA RESOLUCIÓN FINAL PREVISTA EN EL ARTÍCULO 69-B, PÁRRAFO CUARTO, DEL CFF. EL PLAZO PARA INTERPONERLO COMIENZA A PARTIR DE SU NOTIFICACIÓN A TRAVÉS DEL BUZÓN TRIBUTARIO.</t>
+          <t>COMPENSACIÓN ECONÓMICA. ELEMENTOS MÍNIMOS QUE LA PERSONA JUZGADORA DEBE CONSIDERAR PARA MOTIVAR LA RESOLUCIÓN QUE LA CUANTIFICA, CON PERSPECTIVA DE GÉNERO.</t>
         </is>
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>2031931</t>
+          <t>2032154</t>
         </is>
       </c>
       <c r="M94" s="11" t="inlineStr"/>
       <c r="N94" s="11" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
         </is>
       </c>
       <c r="O94" s="11" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — captura automática</t>
         </is>
       </c>
       <c r="P94" s="11" t="inlineStr"/>
       <c r="Q94" s="11" t="inlineStr">
         <is>
-          <t>El plazo de 30 días para interponer recurso de revocación contra resolución definitiva del 69-B se computa desde notificación por buzón tributario, no desde publicación en DOF.</t>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
         </is>
       </c>
       <c r="R94" s="11" t="inlineStr">
         <is>
-          <t>Define cómputo de plazo para defensa contra inclusión definitiva en EFOS.</t>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
         </is>
       </c>
       <c r="S94" s="11" t="inlineStr">
         <is>
-          <t>Hay que monitorear el buzón tributario. Cuenta el plazo desde recepción ahí, no desde publicación DOF. Crítico para no perder defensa.</t>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
         </is>
       </c>
       <c r="T94" s="11" t="inlineStr"/>
       <c r="U94" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031931</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032154</t>
         </is>
       </c>
       <c r="V94" s="11" t="inlineStr">
         <is>
-          <t>69-B CFF · recurso revocación · buzón tributario · EFOS</t>
+          <t>Perspectiva de género · actualización automática</t>
         </is>
       </c>
     </row>
     <row r="95" ht="80" customHeight="1">
       <c r="A95" s="13" t="inlineStr">
         <is>
-          <t>fis-cfd-003</t>
+          <t>auto-2032184</t>
         </is>
       </c>
       <c r="B95" s="13" t="n">
@@ -12531,17 +12531,17 @@
       </c>
       <c r="D95" s="13" t="inlineStr">
         <is>
-          <t>Fiscal</t>
+          <t>Constitucional / DDHH</t>
         </is>
       </c>
       <c r="E95" s="13" t="inlineStr">
         <is>
-          <t>Comprobantes fiscales (CFDI)</t>
+          <t>Perspectiva de género</t>
         </is>
       </c>
       <c r="F95" s="13" t="inlineStr">
         <is>
-          <t>Materialidad — fundar y motivar</t>
+          <t>Actualización automática semanal</t>
         </is>
       </c>
       <c r="G95" s="13" t="inlineStr">
@@ -12566,57 +12566,57 @@
       </c>
       <c r="K95" s="14" t="inlineStr">
         <is>
-          <t>PRESUNCIÓN DE INEXISTENCIA DE OPERACIONES AMPARADAS EN COMPROBANTES FISCALES. DEBER DE FUNDAR Y MOTIVAR LA DECISIÓN DE REVERTIR LA CARGA PROBATORIA PARA ACREDITAR SU MATERIALIDAD.</t>
+          <t>VIOLENCIA FAMILIAR. CUANDO LA VÍCTIMA SEA UNA PERSONA MENOR DE EDAD Y SE ALEGUE ALIENACIÓN O MANIPULACIÓN PARENTAL, EL ÓRGANO JURISDICCIONAL DEBE ORDENAR LA PRÁCTICA DE PRUEBAS PERICIALES PARA VERIFICAR SI SE ACTUALIZA DICHA CONDICIÓN.</t>
         </is>
       </c>
       <c r="L95" s="13" t="inlineStr">
         <is>
-          <t>2031350</t>
+          <t>2032184</t>
         </is>
       </c>
       <c r="M95" s="13" t="inlineStr"/>
       <c r="N95" s="13" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
         </is>
       </c>
       <c r="O95" s="13" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — captura automática</t>
         </is>
       </c>
       <c r="P95" s="13" t="inlineStr"/>
       <c r="Q95" s="13" t="inlineStr">
         <is>
-          <t>El SAT no puede simplemente requerir materialidad; debe fundar y motivar específicamente las razones por las que presume inexistencia. Sin esa fundamentación, la inversión de carga es inválida.</t>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
         </is>
       </c>
       <c r="R95" s="13" t="inlineStr">
         <is>
-          <t>Defensa fuerte para contribuyentes auditados.</t>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
         </is>
       </c>
       <c r="S95" s="13" t="inlineStr">
         <is>
-          <t>Si el SAT no detalla por qué presume inexistencia (red flag específico), su requerimiento es nulo. Cuestionar fundamentación es el primer paso del litigio.</t>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
         </is>
       </c>
       <c r="T95" s="13" t="inlineStr"/>
       <c r="U95" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031350</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032184</t>
         </is>
       </c>
       <c r="V95" s="13" t="inlineStr">
         <is>
-          <t>69-B · materialidad · fundamentación · 12a Época</t>
+          <t>Perspectiva de género · actualización automática</t>
         </is>
       </c>
     </row>
     <row r="96" ht="80" customHeight="1">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>fis-cfd-004</t>
+          <t>amp-gen-001</t>
         </is>
       </c>
       <c r="B96" s="11" t="n">
@@ -12629,17 +12629,17 @@
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>Fiscal</t>
+          <t>Constitucional / DDHH</t>
         </is>
       </c>
       <c r="E96" s="11" t="inlineStr">
         <is>
-          <t>Comprobantes fiscales (CFDI)</t>
+          <t>Perspectiva de género interseccional</t>
         </is>
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>Nulidad EFOS — efectos sobre proveedor</t>
+          <t>Acceso a la justicia para mujeres cuidadoras</t>
         </is>
       </c>
       <c r="G96" s="11" t="inlineStr">
@@ -12664,57 +12664,57 @@
       </c>
       <c r="K96" s="12" t="inlineStr">
         <is>
-          <t>PRESUNCIÓN DE INEXISTENCIA DE OPERACIONES. CONSECUENCIA DE LA NULIDAD DE LA RESOLUCIÓN QUE INCLUYE A UN PROVEEDOR EN EL LISTADO DE EMPRESAS QUE FACTURAN OPERACIONES SIMULADAS (EFOS).</t>
+          <t>ACCESO A LA JUSTICIA EN CONDICIONES DE IGUALDAD SUSTANTIVA. LAS MANIFESTACIONES DE MUJERES QUE AFIRMAN REALIZAR LABORES DE CUIDADO NO REMUNERADAS DEBEN VALORARSE CON PERSPECTIVA DE GÉNERO INTERSECCIONAL.</t>
         </is>
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>2031349</t>
+          <t>2032067</t>
         </is>
       </c>
       <c r="M96" s="11" t="inlineStr"/>
       <c r="N96" s="11" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="O96" s="11" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>SJF 12a Época — VERIFICADO</t>
         </is>
       </c>
       <c r="P96" s="11" t="inlineStr"/>
       <c r="Q96" s="11" t="inlineStr">
         <is>
-          <t>Cuando se obtiene la nulidad de la resolución que incluyó al proveedor en EFOS definitivas, esa nulidad debe surtir efectos respecto del contribuyente que deducción afectada.</t>
+          <t>En procesos donde las mujeres afirman dedicarse a labores de cuidado, sus manifestaciones deben valorarse con perspectiva de género interseccional (considerando clase, edad, etnia, discapacidad y otros factores).</t>
         </is>
       </c>
       <c r="R96" s="11" t="inlineStr">
         <is>
-          <t>Cadena de protección para contribuyentes que dedujeron con proveedores listados.</t>
+          <t>Estándar probatorio favorable para mujeres en juicios civiles, familiares, laborales.</t>
         </is>
       </c>
       <c r="S96" s="11" t="inlineStr">
         <is>
-          <t>Si tu proveedor logra que le quiten de EFOS por sentencia firme, tú puedes invocarlo para recuperar deducciones rechazadas. Defensa colectiva.</t>
+          <t>En alimentos, pensiones, compensación por trabajo doméstico y otros litigios, el juez debe creer y valorar con flexibilidad las declaraciones de mujeres cuidadoras.</t>
         </is>
       </c>
       <c r="T96" s="11" t="inlineStr"/>
       <c r="U96" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031349</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032067</t>
         </is>
       </c>
       <c r="V96" s="11" t="inlineStr">
         <is>
-          <t>EFOS · nulidad · deducciones · 12a Época</t>
+          <t>perspectiva género · interseccional · acceso justicia · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="97" ht="80" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>lab-des-002</t>
+          <t>fis-cfd-002</t>
         </is>
       </c>
       <c r="B97" s="13" t="n">
@@ -12727,27 +12727,27 @@
       </c>
       <c r="D97" s="13" t="inlineStr">
         <is>
-          <t>Laboral</t>
+          <t>Fiscal</t>
         </is>
       </c>
       <c r="E97" s="13" t="inlineStr">
         <is>
-          <t>Despido injustificado</t>
+          <t>Comprobantes fiscales (CFDI)</t>
         </is>
       </c>
       <c r="F97" s="13" t="inlineStr">
         <is>
-          <t>Carga patrón cuando alega rescisión justificada posterior</t>
+          <t>69-B — recurso de revocación y buzón tributario</t>
         </is>
       </c>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>jurisprudencia</t>
         </is>
       </c>
       <c r="H97" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I97" s="13" t="inlineStr">
@@ -12762,18 +12762,18 @@
       </c>
       <c r="K97" s="14" t="inlineStr">
         <is>
-          <t>RELACIÓN LABORAL. CUANDO LA PERSONA TRABAJADORA MANIFIESTA QUE FUE DESPEDIDA INJUSTIFICADAMENTE EN CIERTA FECHA Y EL PATRÓN ARGUMENTA QUE AQUÉLLA SUBSISTIÓ Y QUE POSTERIORMENTE LA RESCINDIÓ DE FORMA JUSTIFICADA, LE CORRESPONDE PROBAR AMBOS HECHOS.</t>
+          <t>RECURSO DE REVOCACIÓN CONTRA LA RESOLUCIÓN FINAL PREVISTA EN EL ARTÍCULO 69-B, PÁRRAFO CUARTO, DEL CFF. EL PLAZO PARA INTERPONERLO COMIENZA A PARTIR DE SU NOTIFICACIÓN A TRAVÉS DEL BUZÓN TRIBUTARIO.</t>
         </is>
       </c>
       <c r="L97" s="13" t="inlineStr">
         <is>
-          <t>2029731</t>
+          <t>2031931</t>
         </is>
       </c>
       <c r="M97" s="13" t="inlineStr"/>
       <c r="N97" s="13" t="inlineStr">
         <is>
-          <t>2024-2025</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O97" s="13" t="inlineStr">
@@ -12784,35 +12784,35 @@
       <c r="P97" s="13" t="inlineStr"/>
       <c r="Q97" s="13" t="inlineStr">
         <is>
-          <t>Si el patrón niega el despido alegado y agrega rescisión justificada posterior, tiene carga de probar AMBOS: que la relación subsistió tras la fecha del supuesto despido y que la rescisión posterior fue justificada.</t>
+          <t>El plazo de 30 días para interponer recurso de revocación contra resolución definitiva del 69-B se computa desde notificación por buzón tributario, no desde publicación en DOF.</t>
         </is>
       </c>
       <c r="R97" s="13" t="inlineStr">
         <is>
-          <t>Carga doble para patrón que cambia versión durante el juicio.</t>
+          <t>Define cómputo de plazo para defensa contra inclusión definitiva en EFOS.</t>
         </is>
       </c>
       <c r="S97" s="13" t="inlineStr">
         <is>
-          <t>Estrategia trabajadora: forzar al patrón a esa narrativa, queda con carga reforzada.</t>
+          <t>Hay que monitorear el buzón tributario. Cuenta el plazo desde recepción ahí, no desde publicación DOF. Crítico para no perder defensa.</t>
         </is>
       </c>
       <c r="T97" s="13" t="inlineStr"/>
       <c r="U97" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029731</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031931</t>
         </is>
       </c>
       <c r="V97" s="13" t="inlineStr">
         <is>
-          <t>despido · rescisión · carga probatoria patrón</t>
+          <t>69-B CFF · recurso revocación · buzón tributario · EFOS</t>
         </is>
       </c>
     </row>
     <row r="98" ht="80" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>lab-ren-001</t>
+          <t>fis-cfd-003</t>
         </is>
       </c>
       <c r="B98" s="11" t="n">
@@ -12825,17 +12825,17 @@
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>Laboral</t>
+          <t>Fiscal</t>
         </is>
       </c>
       <c r="E98" s="11" t="inlineStr">
         <is>
-          <t>Renuncia laboral</t>
+          <t>Comprobantes fiscales (CFDI)</t>
         </is>
       </c>
       <c r="F98" s="11" t="inlineStr">
         <is>
-          <t>Hora de terminación — carga del patrón</t>
+          <t>Materialidad — fundar y motivar</t>
         </is>
       </c>
       <c r="G98" s="11" t="inlineStr">
@@ -12845,7 +12845,7 @@
       </c>
       <c r="H98" s="11" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I98" s="11" t="inlineStr">
@@ -12860,18 +12860,18 @@
       </c>
       <c r="K98" s="12" t="inlineStr">
         <is>
-          <t>RENUNCIA. CORRESPONDE A LA PARTE DEMANDADA PERFECCIONARLA CON ALGÚN MEDIO DE PRUEBA, CUANDO EXISTA CONTROVERSIA RESPECTO DE LA HORA DE TERMINACIÓN DEL VÍNCULO LABORAL Y ÉSTA NO CONSTE EN EL ESCRITO RELATIVO.</t>
+          <t>PRESUNCIÓN DE INEXISTENCIA DE OPERACIONES AMPARADAS EN COMPROBANTES FISCALES. DEBER DE FUNDAR Y MOTIVAR LA DECISIÓN DE REVERTIR LA CARGA PROBATORIA PARA ACREDITAR SU MATERIALIDAD.</t>
         </is>
       </c>
       <c r="L98" s="11" t="inlineStr">
         <is>
-          <t>2028640</t>
+          <t>2031350</t>
         </is>
       </c>
       <c r="M98" s="11" t="inlineStr"/>
       <c r="N98" s="11" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O98" s="11" t="inlineStr">
@@ -12882,35 +12882,35 @@
       <c r="P98" s="11" t="inlineStr"/>
       <c r="Q98" s="11" t="inlineStr">
         <is>
-          <t>Si el patrón ofrece renuncia sin hora exacta y el trabajador alega despido a cierta hora, el patrón debe acreditar con prueba adicional la hora de la renuncia.</t>
+          <t>El SAT no puede simplemente requerir materialidad; debe fundar y motivar específicamente las razones por las que presume inexistencia. Sin esa fundamentación, la inversión de carga es inválida.</t>
         </is>
       </c>
       <c r="R98" s="11" t="inlineStr">
         <is>
-          <t>Cuestionamiento a renuncias forzadas con fechas/horas imprecisas.</t>
+          <t>Defensa fuerte para contribuyentes auditados.</t>
         </is>
       </c>
       <c r="S98" s="11" t="inlineStr">
         <is>
-          <t>Trabajador debe declarar hora exacta del despido; patrón tendrá que probar hora distinta.</t>
+          <t>Si el SAT no detalla por qué presume inexistencia (red flag específico), su requerimiento es nulo. Cuestionar fundamentación es el primer paso del litigio.</t>
         </is>
       </c>
       <c r="T98" s="11" t="inlineStr"/>
       <c r="U98" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2028640</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031350</t>
         </is>
       </c>
       <c r="V98" s="11" t="inlineStr">
         <is>
-          <t>renuncia · hora despido · carga probatoria</t>
+          <t>69-B · materialidad · fundamentación · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="99" ht="80" customHeight="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>lab-ren-002</t>
+          <t>fis-cfd-004</t>
         </is>
       </c>
       <c r="B99" s="13" t="n">
@@ -12923,17 +12923,17 @@
       </c>
       <c r="D99" s="13" t="inlineStr">
         <is>
-          <t>Laboral</t>
+          <t>Fiscal</t>
         </is>
       </c>
       <c r="E99" s="13" t="inlineStr">
         <is>
-          <t>Renuncia laboral</t>
+          <t>Comprobantes fiscales (CFDI)</t>
         </is>
       </c>
       <c r="F99" s="13" t="inlineStr">
         <is>
-          <t>Veracidad — carga reforzada si trabajador iba a jubilarse</t>
+          <t>Nulidad EFOS — efectos sobre proveedor</t>
         </is>
       </c>
       <c r="G99" s="13" t="inlineStr">
@@ -12943,7 +12943,7 @@
       </c>
       <c r="H99" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I99" s="13" t="inlineStr">
@@ -12958,18 +12958,18 @@
       </c>
       <c r="K99" s="14" t="inlineStr">
         <is>
-          <t>RENUNCIA. PARA QUE SEA VEROSÍMIL Y, POR ENDE, TENGA EFICACIA DEMOSTRATIVA PLENA, CORRESPONDE AL PATRÓN PROBAR QUE REÚNE LAS CONDICIONES DE CERTEZA Y LOS ELEMENTOS MÍNIMOS QUE REFLEJEN LA VOLUNTAD, AUTONOMÍA Y ESPONTANEIDAD DEL TRABAJADOR, SI ESTÁ PRÓXIMO A JUBILARSE.</t>
+          <t>PRESUNCIÓN DE INEXISTENCIA DE OPERACIONES. CONSECUENCIA DE LA NULIDAD DE LA RESOLUCIÓN QUE INCLUYE A UN PROVEEDOR EN EL LISTADO DE EMPRESAS QUE FACTURAN OPERACIONES SIMULADAS (EFOS).</t>
         </is>
       </c>
       <c r="L99" s="13" t="inlineStr">
         <is>
-          <t>2027058</t>
+          <t>2031349</t>
         </is>
       </c>
       <c r="M99" s="13" t="inlineStr"/>
       <c r="N99" s="13" t="inlineStr">
         <is>
-          <t>2023-2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O99" s="13" t="inlineStr">
@@ -12980,35 +12980,35 @@
       <c r="P99" s="13" t="inlineStr"/>
       <c r="Q99" s="13" t="inlineStr">
         <is>
-          <t>Cuando el trabajador estaba próximo a adquirir derechos jubilatorios, la renuncia exigida pasa por estándar reforzado de veracidad: voluntad, autonomía y espontaneidad demostradas con prueba sólida.</t>
+          <t>Cuando se obtiene la nulidad de la resolución que incluyó al proveedor en EFOS definitivas, esa nulidad debe surtir efectos respecto del contribuyente que deducción afectada.</t>
         </is>
       </c>
       <c r="R99" s="13" t="inlineStr">
         <is>
-          <t>Protección antes de jubilación: renuncias sospechosas no pasan.</t>
+          <t>Cadena de protección para contribuyentes que dedujeron con proveedores listados.</t>
         </is>
       </c>
       <c r="S99" s="13" t="inlineStr">
         <is>
-          <t>Defensa trabajadora: si estaba a meses/años de jubilarse, atacar renuncia por falta de espontaneidad.</t>
+          <t>Si tu proveedor logra que le quiten de EFOS por sentencia firme, tú puedes invocarlo para recuperar deducciones rechazadas. Defensa colectiva.</t>
         </is>
       </c>
       <c r="T99" s="13" t="inlineStr"/>
       <c r="U99" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027058</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031349</t>
         </is>
       </c>
       <c r="V99" s="13" t="inlineStr">
         <is>
-          <t>renuncia · jubilación · veracidad · carga reforzada</t>
+          <t>EFOS · nulidad · deducciones · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="100" ht="80" customHeight="1">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>sen-020</t>
+          <t>lab-des-002</t>
         </is>
       </c>
       <c r="B100" s="11" t="n">
@@ -13021,27 +13021,27 @@
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>Mercantil</t>
+          <t>Laboral</t>
         </is>
       </c>
       <c r="E100" s="11" t="inlineStr">
         <is>
-          <t>Costas en juicio mercantil — tasación</t>
+          <t>Despido injustificado</t>
         </is>
       </c>
       <c r="F100" s="11" t="inlineStr">
         <is>
-          <t>Línea del Primer y Segundo Circuito (CDMX y Edomex)</t>
+          <t>Carga patrón cuando alega rescisión justificada posterior</t>
         </is>
       </c>
       <c r="G100" s="11" t="inlineStr">
         <is>
-          <t>sentencia hito</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H100" s="11" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I100" s="11" t="inlineStr">
@@ -13051,58 +13051,62 @@
       </c>
       <c r="J100" s="11" t="inlineStr">
         <is>
-          <t>Primer y Segundo Circuito</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="K100" s="12" t="inlineStr">
         <is>
-          <t>Costas mercantiles — base de cuantificación y arancel aplicable</t>
+          <t>RELACIÓN LABORAL. CUANDO LA PERSONA TRABAJADORA MANIFIESTA QUE FUE DESPEDIDA INJUSTIFICADAMENTE EN CIERTA FECHA Y EL PATRÓN ARGUMENTA QUE AQUÉLLA SUBSISTIÓ Y QUE POSTERIORMENTE LA RESCINDIÓ DE FORMA JUSTIFICADA, LE CORRESPONDE PROBAR AMBOS HECHOS.</t>
         </is>
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>Línea de Colegiados — múltiples</t>
+          <t>2029731</t>
         </is>
       </c>
       <c r="M100" s="11" t="inlineStr"/>
       <c r="N100" s="11" t="inlineStr">
         <is>
-          <t>Línea consolidada</t>
-        </is>
-      </c>
-      <c r="O100" s="11" t="inlineStr"/>
+          <t>2024-2025</t>
+        </is>
+      </c>
+      <c r="O100" s="11" t="inlineStr">
+        <is>
+          <t>Gaceta SJF — VERIFICADO</t>
+        </is>
+      </c>
       <c r="P100" s="11" t="inlineStr"/>
       <c r="Q100" s="11" t="inlineStr">
         <is>
-          <t>Las costas en juicio mercantil se cuantifican con base en el monto efectivamente condenado y conforme al arancel local vigente al momento de cuantificarlas. La condena en costas presupone temeridad o vencimiento total.</t>
+          <t>Si el patrón niega el despido alegado y agrega rescisión justificada posterior, tiene carga de probar AMBOS: que la relación subsistió tras la fecha del supuesto despido y que la rescisión posterior fue justificada.</t>
         </is>
       </c>
       <c r="R100" s="11" t="inlineStr">
         <is>
-          <t>Marco práctico para pretensión y oposición a costas.</t>
+          <t>Carga doble para patrón que cambia versión durante el juicio.</t>
         </is>
       </c>
       <c r="S100" s="11" t="inlineStr">
         <is>
-          <t>El acreedor que gana en ejecutivo debe solicitar tasación con arancel actualizado. El deudor debe oponerse cuando la cuantificación excede el monto del juicio o aplica arancel inadecuado.</t>
+          <t>Estrategia trabajadora: forzar al patrón a esa narrativa, queda con carga reforzada.</t>
         </is>
       </c>
       <c r="T100" s="11" t="inlineStr"/>
       <c r="U100" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031803</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2029731</t>
         </is>
       </c>
       <c r="V100" s="11" t="inlineStr">
         <is>
-          <t>costas · tasación · arancel · mercantil</t>
+          <t>despido · rescisión · carga probatoria patrón</t>
         </is>
       </c>
     </row>
     <row r="101" ht="80" customHeight="1">
       <c r="A101" s="13" t="inlineStr">
         <is>
-          <t>mer-eje-002</t>
+          <t>lab-ren-001</t>
         </is>
       </c>
       <c r="B101" s="13" t="n">
@@ -13115,22 +13119,22 @@
       </c>
       <c r="D101" s="13" t="inlineStr">
         <is>
-          <t>Mercantil</t>
+          <t>Laboral</t>
         </is>
       </c>
       <c r="E101" s="13" t="inlineStr">
         <is>
-          <t>Juicio ejecutivo mercantil</t>
+          <t>Renuncia laboral</t>
         </is>
       </c>
       <c r="F101" s="13" t="inlineStr">
         <is>
-          <t>Improcedencia — análisis oficioso en amparo directo</t>
+          <t>Hora de terminación — carga del patrón</t>
         </is>
       </c>
       <c r="G101" s="13" t="inlineStr">
         <is>
-          <t>jurisprudencia</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H101" s="13" t="inlineStr">
@@ -13150,18 +13154,18 @@
       </c>
       <c r="K101" s="14" t="inlineStr">
         <is>
-          <t>IMPROCEDENCIA DE LA VÍA EJECUTIVA MERCANTIL. AL TRATARSE DE UN PRESUPUESTO PROCESAL, PUEDE ANALIZARSE DE OFICIO EN EL JUICIO DE AMPARO DIRECTO.</t>
+          <t>RENUNCIA. CORRESPONDE A LA PARTE DEMANDADA PERFECCIONARLA CON ALGÚN MEDIO DE PRUEBA, CUANDO EXISTA CONTROVERSIA RESPECTO DE LA HORA DE TERMINACIÓN DEL VÍNCULO LABORAL Y ÉSTA NO CONSTE EN EL ESCRITO RELATIVO.</t>
         </is>
       </c>
       <c r="L101" s="13" t="inlineStr">
         <is>
-          <t>2025924</t>
+          <t>2028640</t>
         </is>
       </c>
       <c r="M101" s="13" t="inlineStr"/>
       <c r="N101" s="13" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="O101" s="13" t="inlineStr">
@@ -13172,35 +13176,35 @@
       <c r="P101" s="13" t="inlineStr"/>
       <c r="Q101" s="13" t="inlineStr">
         <is>
-          <t>La improcedencia de la vía ejecutiva mercantil es presupuesto procesal y puede analizarse de oficio incluso en amparo directo, aunque las instancias previas no lo hayan abordado a fondo.</t>
+          <t>Si el patrón ofrece renuncia sin hora exacta y el trabajador alega despido a cierta hora, el patrón debe acreditar con prueba adicional la hora de la renuncia.</t>
         </is>
       </c>
       <c r="R101" s="13" t="inlineStr">
         <is>
-          <t>Defensa de última instancia para deudores ejecutados con documentos viciados.</t>
+          <t>Cuestionamiento a renuncias forzadas con fechas/horas imprecisas.</t>
         </is>
       </c>
       <c r="S101" s="13" t="inlineStr">
         <is>
-          <t>Aun perdiendo en primera y segunda instancia, en amparo directo se puede plantear.</t>
+          <t>Trabajador debe declarar hora exacta del despido; patrón tendrá que probar hora distinta.</t>
         </is>
       </c>
       <c r="T101" s="13" t="inlineStr"/>
       <c r="U101" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2025924</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2028640</t>
         </is>
       </c>
       <c r="V101" s="13" t="inlineStr">
         <is>
-          <t>vía ejecutiva mercantil · amparo directo · oficio</t>
+          <t>renuncia · hora despido · carga probatoria</t>
         </is>
       </c>
     </row>
     <row r="102" ht="80" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>mer-eje-003</t>
+          <t>lab-ren-002</t>
         </is>
       </c>
       <c r="B102" s="11" t="n">
@@ -13213,17 +13217,17 @@
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>Mercantil</t>
+          <t>Laboral</t>
         </is>
       </c>
       <c r="E102" s="11" t="inlineStr">
         <is>
-          <t>Juicio ejecutivo mercantil</t>
+          <t>Renuncia laboral</t>
         </is>
       </c>
       <c r="F102" s="11" t="inlineStr">
         <is>
-          <t>Mora — fecha de actualización</t>
+          <t>Veracidad — carga reforzada si trabajador iba a jubilarse</t>
         </is>
       </c>
       <c r="G102" s="11" t="inlineStr">
@@ -13233,7 +13237,7 @@
       </c>
       <c r="H102" s="11" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I102" s="11" t="inlineStr">
@@ -13248,57 +13252,57 @@
       </c>
       <c r="K102" s="12" t="inlineStr">
         <is>
-          <t>MORA EN EL JUICIO EJECUTIVO MERCANTIL. SE ACTUALIZA CON MOTIVO DE LA INTERPELACIÓN FORMULADA EN EL EMPLAZAMIENTO Y NO EN LA FECHA DE VENCIMIENTO ESTABLECIDA EN EL PAGARÉ BASE DE LA ACCIÓN.</t>
+          <t>RENUNCIA. PARA QUE SEA VEROSÍMIL Y, POR ENDE, TENGA EFICACIA DEMOSTRATIVA PLENA, CORRESPONDE AL PATRÓN PROBAR QUE REÚNE LAS CONDICIONES DE CERTEZA Y LOS ELEMENTOS MÍNIMOS QUE REFLEJEN LA VOLUNTAD, AUTONOMÍA Y ESPONTANEIDAD DEL TRABAJADOR, SI ESTÁ PRÓXIMO A JUBILARSE.</t>
         </is>
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>2031591</t>
+          <t>2027058</t>
         </is>
       </c>
       <c r="M102" s="11" t="inlineStr"/>
       <c r="N102" s="11" t="inlineStr">
         <is>
-          <t>2025-2026</t>
+          <t>2023-2024</t>
         </is>
       </c>
       <c r="O102" s="11" t="inlineStr">
         <is>
-          <t>SJF 12a Época — VERIFICADO</t>
+          <t>Gaceta SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P102" s="11" t="inlineStr"/>
       <c r="Q102" s="11" t="inlineStr">
         <is>
-          <t>Cuando el pagaré señala genéricamente como lugar de pago una ciudad, la mora no se actualiza con el vencimiento sino con la interpelación en el emplazamiento judicial.</t>
+          <t>Cuando el trabajador estaba próximo a adquirir derechos jubilatorios, la renuncia exigida pasa por estándar reforzado de veracidad: voluntad, autonomía y espontaneidad demostradas con prueba sólida.</t>
         </is>
       </c>
       <c r="R102" s="11" t="inlineStr">
         <is>
-          <t>Define desde cuándo corren intereses moratorios.</t>
+          <t>Protección antes de jubilación: renuncias sospechosas no pasan.</t>
         </is>
       </c>
       <c r="S102" s="11" t="inlineStr">
         <is>
-          <t>Pagarés con lugar genérico: los intereses moratorios corren desde emplazamiento, no desde vencimiento.</t>
+          <t>Defensa trabajadora: si estaba a meses/años de jubilarse, atacar renuncia por falta de espontaneidad.</t>
         </is>
       </c>
       <c r="T102" s="11" t="inlineStr"/>
       <c r="U102" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031591</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027058</t>
         </is>
       </c>
       <c r="V102" s="11" t="inlineStr">
         <is>
-          <t>mora · intereses moratorios · interpelación · 12a Época</t>
+          <t>renuncia · jubilación · veracidad · carga reforzada</t>
         </is>
       </c>
     </row>
     <row r="103" ht="80" customHeight="1">
       <c r="A103" s="13" t="inlineStr">
         <is>
-          <t>mer-pag-002</t>
+          <t>sen-020</t>
         </is>
       </c>
       <c r="B103" s="13" t="n">
@@ -13316,22 +13320,22 @@
       </c>
       <c r="E103" s="13" t="inlineStr">
         <is>
-          <t>Títulos de crédito — pagaré</t>
+          <t>Costas en juicio mercantil — tasación</t>
         </is>
       </c>
       <c r="F103" s="13" t="inlineStr">
         <is>
-          <t>Acción causal — pagaré como prueba del contrato</t>
+          <t>Línea del Primer y Segundo Circuito (CDMX y Edomex)</t>
         </is>
       </c>
       <c r="G103" s="13" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>sentencia hito</t>
         </is>
       </c>
       <c r="H103" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I103" s="13" t="inlineStr">
@@ -13341,62 +13345,58 @@
       </c>
       <c r="J103" s="13" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Primer y Segundo Circuito</t>
         </is>
       </c>
       <c r="K103" s="14" t="inlineStr">
         <is>
-          <t>ACCIÓN CAUSAL. SU EJERCICIO PARA EL COBRO DE UN TÍTULO DE CRÉDITO PUEDE SUSTENTARSE EN EL CONTRATO CONTENIDO EN EL PAGARÉ, DERIVADO DEL OTORGAMIENTO DE UN PRÉSTAMO A CORTO PLAZO.</t>
+          <t>Costas mercantiles — base de cuantificación y arancel aplicable</t>
         </is>
       </c>
       <c r="L103" s="13" t="inlineStr">
         <is>
-          <t>2024056</t>
+          <t>Línea de Colegiados — múltiples</t>
         </is>
       </c>
       <c r="M103" s="13" t="inlineStr"/>
       <c r="N103" s="13" t="inlineStr">
         <is>
-          <t>2022</t>
-        </is>
-      </c>
-      <c r="O103" s="13" t="inlineStr">
-        <is>
-          <t>Gaceta SJF — VERIFICADO</t>
-        </is>
-      </c>
+          <t>Línea consolidada</t>
+        </is>
+      </c>
+      <c r="O103" s="13" t="inlineStr"/>
       <c r="P103" s="13" t="inlineStr"/>
       <c r="Q103" s="13" t="inlineStr">
         <is>
-          <t>Si el pagaré pierde eficacia ejecutiva o el acreedor decide no usar la vía ejecutiva, puede ejercer acción causal con el pagaré como prueba documental del contrato subyacente.</t>
+          <t>Las costas en juicio mercantil se cuantifican con base en el monto efectivamente condenado y conforme al arancel local vigente al momento de cuantificarlas. La condena en costas presupone temeridad o vencimiento total.</t>
         </is>
       </c>
       <c r="R103" s="13" t="inlineStr">
         <is>
-          <t>Salvavidas para acreedores cuando el pagaré tiene vicios formales.</t>
+          <t>Marco práctico para pretensión y oposición a costas.</t>
         </is>
       </c>
       <c r="S103" s="13" t="inlineStr">
         <is>
-          <t>Si no procede el ejecutivo, vía ordinaria con el pagaré como documental.</t>
+          <t>El acreedor que gana en ejecutivo debe solicitar tasación con arancel actualizado. El deudor debe oponerse cuando la cuantificación excede el monto del juicio o aplica arancel inadecuado.</t>
         </is>
       </c>
       <c r="T103" s="13" t="inlineStr"/>
       <c r="U103" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024056</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031803</t>
         </is>
       </c>
       <c r="V103" s="13" t="inlineStr">
         <is>
-          <t>pagaré · acción causal · ordinario mercantil</t>
+          <t>costas · tasación · arancel · mercantil</t>
         </is>
       </c>
     </row>
     <row r="104" ht="80" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>mer-pag-003</t>
+          <t>mer-eje-002</t>
         </is>
       </c>
       <c r="B104" s="11" t="n">
@@ -13414,22 +13414,22 @@
       </c>
       <c r="E104" s="11" t="inlineStr">
         <is>
-          <t>Títulos de crédito — pagaré</t>
+          <t>Juicio ejecutivo mercantil</t>
         </is>
       </c>
       <c r="F104" s="11" t="inlineStr">
         <is>
-          <t>Pagarés seriados — lugar de pago</t>
+          <t>Improcedencia — análisis oficioso en amparo directo</t>
         </is>
       </c>
       <c r="G104" s="11" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>jurisprudencia</t>
         </is>
       </c>
       <c r="H104" s="11" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I104" s="11" t="inlineStr">
@@ -13444,18 +13444,18 @@
       </c>
       <c r="K104" s="12" t="inlineStr">
         <is>
-          <t>PAGARÉS SERIADOS. ANTE LA AUSENCIA DE "LUGAR DE PAGO" EN UNO DE ÉSTOS, DEBE ATENDERSE A LO PACTADO EN OTRO DIVERSO DONDE SÍ SE SEÑALÓ.</t>
+          <t>IMPROCEDENCIA DE LA VÍA EJECUTIVA MERCANTIL. AL TRATARSE DE UN PRESUPUESTO PROCESAL, PUEDE ANALIZARSE DE OFICIO EN EL JUICIO DE AMPARO DIRECTO.</t>
         </is>
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>2019464</t>
+          <t>2025924</t>
         </is>
       </c>
       <c r="M104" s="11" t="inlineStr"/>
       <c r="N104" s="11" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="O104" s="11" t="inlineStr">
@@ -13466,35 +13466,35 @@
       <c r="P104" s="11" t="inlineStr"/>
       <c r="Q104" s="11" t="inlineStr">
         <is>
-          <t>Cuando se emiten varios pagarés seriados y solo uno tiene lugar de pago expreso, ese lugar aplica a toda la serie por integración.</t>
+          <t>La improcedencia de la vía ejecutiva mercantil es presupuesto procesal y puede analizarse de oficio incluso en amparo directo, aunque las instancias previas no lo hayan abordado a fondo.</t>
         </is>
       </c>
       <c r="R104" s="11" t="inlineStr">
         <is>
-          <t>Importante en mutuos con tabla de pagos a 12, 24 o 36 meses.</t>
+          <t>Defensa de última instancia para deudores ejecutados con documentos viciados.</t>
         </is>
       </c>
       <c r="S104" s="11" t="inlineStr">
         <is>
-          <t>Defensa contra excepción de pagaré sin lugar de pago en serie.</t>
+          <t>Aun perdiendo en primera y segunda instancia, en amparo directo se puede plantear.</t>
         </is>
       </c>
       <c r="T104" s="11" t="inlineStr"/>
       <c r="U104" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2019464</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2025924</t>
         </is>
       </c>
       <c r="V104" s="11" t="inlineStr">
         <is>
-          <t>pagaré · pagarés seriados · lugar de pago</t>
+          <t>vía ejecutiva mercantil · amparo directo · oficio</t>
         </is>
       </c>
     </row>
     <row r="105" ht="80" customHeight="1">
       <c r="A105" s="13" t="inlineStr">
         <is>
-          <t>pen-cad-002</t>
+          <t>mer-eje-003</t>
         </is>
       </c>
       <c r="B105" s="13" t="n">
@@ -13507,27 +13507,27 @@
       </c>
       <c r="D105" s="13" t="inlineStr">
         <is>
-          <t>Penal</t>
+          <t>Mercantil</t>
         </is>
       </c>
       <c r="E105" s="13" t="inlineStr">
         <is>
-          <t>Cadena de custodia</t>
+          <t>Juicio ejecutivo mercantil</t>
         </is>
       </c>
       <c r="F105" s="13" t="inlineStr">
         <is>
-          <t>Responsabilidad de la Fiscalía aun con datos del inculpado</t>
+          <t>Mora — fecha de actualización</t>
         </is>
       </c>
       <c r="G105" s="13" t="inlineStr">
         <is>
-          <t>jurisprudencia</t>
+          <t>tesis aislada</t>
         </is>
       </c>
       <c r="H105" s="13" t="inlineStr">
         <is>
-          <t>Undécima Época</t>
+          <t>Duodécima Época</t>
         </is>
       </c>
       <c r="I105" s="13" t="inlineStr">
@@ -13542,57 +13542,57 @@
       </c>
       <c r="K105" s="14" t="inlineStr">
         <is>
-          <t>CADENA DE CUSTODIA. ES RESPONSABILIDAD EXCLUSIVA DE LOS SERVIDORES PÚBLICOS DE LA FISCALÍA, INCLUSO RESPECTO DE DATOS O MEDIOS DE PRUEBA APORTADOS POR EL INCULPADO O SU DEFENSA.</t>
+          <t>MORA EN EL JUICIO EJECUTIVO MERCANTIL. SE ACTUALIZA CON MOTIVO DE LA INTERPELACIÓN FORMULADA EN EL EMPLAZAMIENTO Y NO EN LA FECHA DE VENCIMIENTO ESTABLECIDA EN EL PAGARÉ BASE DE LA ACCIÓN.</t>
         </is>
       </c>
       <c r="L105" s="13" t="inlineStr">
         <is>
-          <t>2027962</t>
+          <t>2031591</t>
         </is>
       </c>
       <c r="M105" s="13" t="inlineStr"/>
       <c r="N105" s="13" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2025-2026</t>
         </is>
       </c>
       <c r="O105" s="13" t="inlineStr">
         <is>
-          <t>Gaceta SJF — VERIFICADO</t>
+          <t>SJF 12a Época — VERIFICADO</t>
         </is>
       </c>
       <c r="P105" s="13" t="inlineStr"/>
       <c r="Q105" s="13" t="inlineStr">
         <is>
-          <t>Conforme al CNPP, la cadena de custodia recae siempre en la Fiscalía, incluso respecto de evidencia aportada por la defensa. La defensa NO carga con su preservación; el MP debe registrarla y custodiarla.</t>
+          <t>Cuando el pagaré señala genéricamente como lugar de pago una ciudad, la mora no se actualiza con el vencimiento sino con la interpelación en el emplazamiento judicial.</t>
         </is>
       </c>
       <c r="R105" s="13" t="inlineStr">
         <is>
-          <t>Reforma carga: la defensa puede aportar evidencia sin temor a romper cadena.</t>
+          <t>Define desde cuándo corren intereses moratorios.</t>
         </is>
       </c>
       <c r="S105" s="13" t="inlineStr">
         <is>
-          <t>Defensa puede aportar peritajes, fotos, audios sin asumir custodia formal.</t>
+          <t>Pagarés con lugar genérico: los intereses moratorios corren desde emplazamiento, no desde vencimiento.</t>
         </is>
       </c>
       <c r="T105" s="13" t="inlineStr"/>
       <c r="U105" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027962</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2031591</t>
         </is>
       </c>
       <c r="V105" s="13" t="inlineStr">
         <is>
-          <t>cadena custodia · CNPP · Fiscalía · evidencia defensa</t>
+          <t>mora · intereses moratorios · interpelación · 12a Época</t>
         </is>
       </c>
     </row>
     <row r="106" ht="80" customHeight="1">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>pen-cad-003</t>
+          <t>mer-pag-002</t>
         </is>
       </c>
       <c r="B106" s="11" t="n">
@@ -13605,17 +13605,17 @@
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>Penal</t>
+          <t>Mercantil</t>
         </is>
       </c>
       <c r="E106" s="11" t="inlineStr">
         <is>
-          <t>Cadena de custodia</t>
+          <t>Títulos de crédito — pagaré</t>
         </is>
       </c>
       <c r="F106" s="11" t="inlineStr">
         <is>
-          <t>Transgresión no torna ilícita la prueba</t>
+          <t>Acción causal — pagaré como prueba del contrato</t>
         </is>
       </c>
       <c r="G106" s="11" t="inlineStr">
@@ -13625,7 +13625,7 @@
       </c>
       <c r="H106" s="11" t="inlineStr">
         <is>
-          <t>Décima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I106" s="11" t="inlineStr">
@@ -13640,18 +13640,18 @@
       </c>
       <c r="K106" s="12" t="inlineStr">
         <is>
-          <t>CADENA DE CUSTODIA. SU TRANSGRESIÓN NO TORNA ILÍCITOS LOS DATOS DE PRUEBA.</t>
+          <t>ACCIÓN CAUSAL. SU EJERCICIO PARA EL COBRO DE UN TÍTULO DE CRÉDITO PUEDE SUSTENTARSE EN EL CONTRATO CONTENIDO EN EL PAGARÉ, DERIVADO DEL OTORGAMIENTO DE UN PRÉSTAMO A CORTO PLAZO.</t>
         </is>
       </c>
       <c r="L106" s="11" t="inlineStr">
         <is>
-          <t>2021845</t>
+          <t>2024056</t>
         </is>
       </c>
       <c r="M106" s="11" t="inlineStr"/>
       <c r="N106" s="11" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="O106" s="11" t="inlineStr">
@@ -13662,35 +13662,35 @@
       <c r="P106" s="11" t="inlineStr"/>
       <c r="Q106" s="11" t="inlineStr">
         <is>
-          <t>La ruptura de cadena de custodia NO convierte automáticamente en ilícita la prueba; solo afecta su valor probatorio. El juez debe ponderar la magnitud de la ruptura.</t>
+          <t>Si el pagaré pierde eficacia ejecutiva o el acreedor decide no usar la vía ejecutiva, puede ejercer acción causal con el pagaré como prueba documental del contrato subyacente.</t>
         </is>
       </c>
       <c r="R106" s="11" t="inlineStr">
         <is>
-          <t>Matiza la regla de exclusión: cadena rota = valor probatorio reducido, no exclusión.</t>
+          <t>Salvavidas para acreedores cuando el pagaré tiene vicios formales.</t>
         </is>
       </c>
       <c r="S106" s="11" t="inlineStr">
         <is>
-          <t>Defensa: argumentar valor cero por ruptura. Acusación: defender la prueba a pesar de la ruptura.</t>
+          <t>Si no procede el ejecutivo, vía ordinaria con el pagaré como documental.</t>
         </is>
       </c>
       <c r="T106" s="11" t="inlineStr"/>
       <c r="U106" s="11" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2021845</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2024056</t>
         </is>
       </c>
       <c r="V106" s="11" t="inlineStr">
         <is>
-          <t>cadena custodia · valor probatorio · exclusión</t>
+          <t>pagaré · acción causal · ordinario mercantil</t>
         </is>
       </c>
     </row>
     <row r="107" ht="80" customHeight="1">
       <c r="A107" s="13" t="inlineStr">
         <is>
-          <t>pen-ppo-001</t>
+          <t>mer-pag-003</t>
         </is>
       </c>
       <c r="B107" s="13" t="n">
@@ -13703,17 +13703,17 @@
       </c>
       <c r="D107" s="13" t="inlineStr">
         <is>
-          <t>Penal</t>
+          <t>Mercantil</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr">
         <is>
-          <t>Prisión preventiva oficiosa</t>
+          <t>Títulos de crédito — pagaré</t>
         </is>
       </c>
       <c r="F107" s="13" t="inlineStr">
         <is>
-          <t>Víctima — falta de legitimación para impugnar cese</t>
+          <t>Pagarés seriados — lugar de pago</t>
         </is>
       </c>
       <c r="G107" s="13" t="inlineStr">
@@ -13723,7 +13723,7 @@
       </c>
       <c r="H107" s="13" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Décima Época</t>
         </is>
       </c>
       <c r="I107" s="13" t="inlineStr">
@@ -13738,57 +13738,57 @@
       </c>
       <c r="K107" s="14" t="inlineStr">
         <is>
-          <t>PRISIÓN PREVENTIVA OFICIOSA. LA VÍCTIMA U OFENDIDO DEL DELITO CARECE DE LEGITIMACIÓN PARA IMPUGNAR EN SEDE CONSTITUCIONAL SU CESE, AL NO TENER INCORPORADA A SU ESFERA JURÍDICA ALGÚN DERECHO QUE LA FACULTE.</t>
+          <t>PAGARÉS SERIADOS. ANTE LA AUSENCIA DE "LUGAR DE PAGO" EN UNO DE ÉSTOS, DEBE ATENDERSE A LO PACTADO EN OTRO DIVERSO DONDE SÍ SE SEÑALÓ.</t>
         </is>
       </c>
       <c r="L107" s="13" t="inlineStr">
         <is>
-          <t>2032107</t>
+          <t>2019464</t>
         </is>
       </c>
       <c r="M107" s="13" t="inlineStr"/>
       <c r="N107" s="13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="O107" s="13" t="inlineStr">
         <is>
-          <t>SJF 12a Época — VERIFICADO</t>
+          <t>Gaceta SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P107" s="13" t="inlineStr"/>
       <c r="Q107" s="13" t="inlineStr">
         <is>
-          <t>La víctima no puede impugnar por amparo la liberación del imputado cuando se cesa la PPO. No hay derecho subjetivo a que el imputado permanezca en prisión preventiva.</t>
+          <t>Cuando se emiten varios pagarés seriados y solo uno tiene lugar de pago expreso, ese lugar aplica a toda la serie por integración.</t>
         </is>
       </c>
       <c r="R107" s="13" t="inlineStr">
         <is>
-          <t>Restringe vía de víctima contra liberaciones por exceso de plazo.</t>
+          <t>Importante en mutuos con tabla de pagos a 12, 24 o 36 meses.</t>
         </is>
       </c>
       <c r="S107" s="13" t="inlineStr">
         <is>
-          <t>Tras PPO cesada (más de 2 años sin sentencia, por ejemplo), la víctima no puede ampararse. Su vía es civil/coadyuvancia para impulsar el proceso, no constitucional.</t>
+          <t>Defensa contra excepción de pagaré sin lugar de pago en serie.</t>
         </is>
       </c>
       <c r="T107" s="13" t="inlineStr"/>
       <c r="U107" s="13" t="inlineStr">
         <is>
-          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032107</t>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2019464</t>
         </is>
       </c>
       <c r="V107" s="13" t="inlineStr">
         <is>
-          <t>PPO · víctima · legitimación · 12a Época</t>
+          <t>pagaré · pagarés seriados · lugar de pago</t>
         </is>
       </c>
     </row>
     <row r="108" ht="80" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>pen-ppo-002</t>
+          <t>pen-cad-002</t>
         </is>
       </c>
       <c r="B108" s="11" t="n">
@@ -13806,22 +13806,22 @@
       </c>
       <c r="E108" s="11" t="inlineStr">
         <is>
-          <t>Prisión preventiva oficiosa</t>
+          <t>Cadena de custodia</t>
         </is>
       </c>
       <c r="F108" s="11" t="inlineStr">
         <is>
-          <t>Cese cuando MP no prueba prolongación</t>
+          <t>Responsabilidad de la Fiscalía aun con datos del inculpado</t>
         </is>
       </c>
       <c r="G108" s="11" t="inlineStr">
         <is>
-          <t>tesis aislada</t>
+          <t>jurisprudencia</t>
         </is>
       </c>
       <c r="H108" s="11" t="inlineStr">
         <is>
-          <t>Duodécima Época</t>
+          <t>Undécima Época</t>
         </is>
       </c>
       <c r="I108" s="11" t="inlineStr">
@@ -13836,55 +13836,349 @@
       </c>
       <c r="K108" s="12" t="inlineStr">
         <is>
-          <t>PRISIÓN PREVENTIVA OFICIOSA. SU CESE ORDENADO CUANDO EL MINISTERIO PÚBLICO NO PRUEBA NI JUSTIFICA SU PROLONGACIÓN, PARA EFECTOS DE QUE SE DEBATA LA IMPOSICIÓN DE OTRAS MEDIDAS CAUTELARES MENOS RESTRICTIVAS.</t>
+          <t>CADENA DE CUSTODIA. ES RESPONSABILIDAD EXCLUSIVA DE LOS SERVIDORES PÚBLICOS DE LA FISCALÍA, INCLUSO RESPECTO DE DATOS O MEDIOS DE PRUEBA APORTADOS POR EL INCULPADO O SU DEFENSA.</t>
         </is>
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>2032108</t>
+          <t>2027962</t>
         </is>
       </c>
       <c r="M108" s="11" t="inlineStr"/>
       <c r="N108" s="11" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="O108" s="11" t="inlineStr">
         <is>
-          <t>SJF 12a Época — VERIFICADO</t>
+          <t>Gaceta SJF — VERIFICADO</t>
         </is>
       </c>
       <c r="P108" s="11" t="inlineStr"/>
       <c r="Q108" s="11" t="inlineStr">
         <is>
-          <t>Al solicitar prolongación de PPO, el MP tiene carga probatoria. Si no la cumple, el juez debe cesar la PPO y reabrir debate sobre medidas cautelares alternativas.</t>
+          <t>Conforme al CNPP, la cadena de custodia recae siempre en la Fiscalía, incluso respecto de evidencia aportada por la defensa. La defensa NO carga con su preservación; el MP debe registrarla y custodiarla.</t>
         </is>
       </c>
       <c r="R108" s="11" t="inlineStr">
         <is>
-          <t>Defensa decisiva contra prolongación automática de PPO.</t>
+          <t>Reforma carga: la defensa puede aportar evidencia sin temor a romper cadena.</t>
         </is>
       </c>
       <c r="S108" s="11" t="inlineStr">
         <is>
-          <t>Cuando MP solicita prolongación sin justificar, la defensa debe exigir prueba concreta. Sin ella, opera el cese y se debate medida alterna (caución, brazalete, presentación periódica).</t>
+          <t>Defensa puede aportar peritajes, fotos, audios sin asumir custodia formal.</t>
         </is>
       </c>
       <c r="T108" s="11" t="inlineStr"/>
       <c r="U108" s="11" t="inlineStr">
         <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2027962</t>
+        </is>
+      </c>
+      <c r="V108" s="11" t="inlineStr">
+        <is>
+          <t>cadena custodia · CNPP · Fiscalía · evidencia defensa</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="80" customHeight="1">
+      <c r="A109" s="13" t="inlineStr">
+        <is>
+          <t>pen-cad-003</t>
+        </is>
+      </c>
+      <c r="B109" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C109" s="13" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D109" s="13" t="inlineStr">
+        <is>
+          <t>Penal</t>
+        </is>
+      </c>
+      <c r="E109" s="13" t="inlineStr">
+        <is>
+          <t>Cadena de custodia</t>
+        </is>
+      </c>
+      <c r="F109" s="13" t="inlineStr">
+        <is>
+          <t>Transgresión no torna ilícita la prueba</t>
+        </is>
+      </c>
+      <c r="G109" s="13" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H109" s="13" t="inlineStr">
+        <is>
+          <t>Décima Época</t>
+        </is>
+      </c>
+      <c r="I109" s="13" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J109" s="13" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K109" s="14" t="inlineStr">
+        <is>
+          <t>CADENA DE CUSTODIA. SU TRANSGRESIÓN NO TORNA ILÍCITOS LOS DATOS DE PRUEBA.</t>
+        </is>
+      </c>
+      <c r="L109" s="13" t="inlineStr">
+        <is>
+          <t>2021845</t>
+        </is>
+      </c>
+      <c r="M109" s="13" t="inlineStr"/>
+      <c r="N109" s="13" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="O109" s="13" t="inlineStr">
+        <is>
+          <t>Gaceta SJF — VERIFICADO</t>
+        </is>
+      </c>
+      <c r="P109" s="13" t="inlineStr"/>
+      <c r="Q109" s="13" t="inlineStr">
+        <is>
+          <t>La ruptura de cadena de custodia NO convierte automáticamente en ilícita la prueba; solo afecta su valor probatorio. El juez debe ponderar la magnitud de la ruptura.</t>
+        </is>
+      </c>
+      <c r="R109" s="13" t="inlineStr">
+        <is>
+          <t>Matiza la regla de exclusión: cadena rota = valor probatorio reducido, no exclusión.</t>
+        </is>
+      </c>
+      <c r="S109" s="13" t="inlineStr">
+        <is>
+          <t>Defensa: argumentar valor cero por ruptura. Acusación: defender la prueba a pesar de la ruptura.</t>
+        </is>
+      </c>
+      <c r="T109" s="13" t="inlineStr"/>
+      <c r="U109" s="13" t="inlineStr">
+        <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2021845</t>
+        </is>
+      </c>
+      <c r="V109" s="13" t="inlineStr">
+        <is>
+          <t>cadena custodia · valor probatorio · exclusión</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="80" customHeight="1">
+      <c r="A110" s="11" t="inlineStr">
+        <is>
+          <t>pen-ppo-001</t>
+        </is>
+      </c>
+      <c r="B110" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" s="11" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D110" s="11" t="inlineStr">
+        <is>
+          <t>Penal</t>
+        </is>
+      </c>
+      <c r="E110" s="11" t="inlineStr">
+        <is>
+          <t>Prisión preventiva oficiosa</t>
+        </is>
+      </c>
+      <c r="F110" s="11" t="inlineStr">
+        <is>
+          <t>Víctima — falta de legitimación para impugnar cese</t>
+        </is>
+      </c>
+      <c r="G110" s="11" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H110" s="11" t="inlineStr">
+        <is>
+          <t>Duodécima Época</t>
+        </is>
+      </c>
+      <c r="I110" s="11" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J110" s="11" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K110" s="12" t="inlineStr">
+        <is>
+          <t>PRISIÓN PREVENTIVA OFICIOSA. LA VÍCTIMA U OFENDIDO DEL DELITO CARECE DE LEGITIMACIÓN PARA IMPUGNAR EN SEDE CONSTITUCIONAL SU CESE, AL NO TENER INCORPORADA A SU ESFERA JURÍDICA ALGÚN DERECHO QUE LA FACULTE.</t>
+        </is>
+      </c>
+      <c r="L110" s="11" t="inlineStr">
+        <is>
+          <t>2032107</t>
+        </is>
+      </c>
+      <c r="M110" s="11" t="inlineStr"/>
+      <c r="N110" s="11" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="O110" s="11" t="inlineStr">
+        <is>
+          <t>SJF 12a Época — VERIFICADO</t>
+        </is>
+      </c>
+      <c r="P110" s="11" t="inlineStr"/>
+      <c r="Q110" s="11" t="inlineStr">
+        <is>
+          <t>La víctima no puede impugnar por amparo la liberación del imputado cuando se cesa la PPO. No hay derecho subjetivo a que el imputado permanezca en prisión preventiva.</t>
+        </is>
+      </c>
+      <c r="R110" s="11" t="inlineStr">
+        <is>
+          <t>Restringe vía de víctima contra liberaciones por exceso de plazo.</t>
+        </is>
+      </c>
+      <c r="S110" s="11" t="inlineStr">
+        <is>
+          <t>Tras PPO cesada (más de 2 años sin sentencia, por ejemplo), la víctima no puede ampararse. Su vía es civil/coadyuvancia para impulsar el proceso, no constitucional.</t>
+        </is>
+      </c>
+      <c r="T110" s="11" t="inlineStr"/>
+      <c r="U110" s="11" t="inlineStr">
+        <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032107</t>
+        </is>
+      </c>
+      <c r="V110" s="11" t="inlineStr">
+        <is>
+          <t>PPO · víctima · legitimación · 12a Época</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="80" customHeight="1">
+      <c r="A111" s="13" t="inlineStr">
+        <is>
+          <t>pen-ppo-002</t>
+        </is>
+      </c>
+      <c r="B111" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C111" s="13" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D111" s="13" t="inlineStr">
+        <is>
+          <t>Penal</t>
+        </is>
+      </c>
+      <c r="E111" s="13" t="inlineStr">
+        <is>
+          <t>Prisión preventiva oficiosa</t>
+        </is>
+      </c>
+      <c r="F111" s="13" t="inlineStr">
+        <is>
+          <t>Cese cuando MP no prueba prolongación</t>
+        </is>
+      </c>
+      <c r="G111" s="13" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t>Duodécima Época</t>
+        </is>
+      </c>
+      <c r="I111" s="13" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J111" s="13" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K111" s="14" t="inlineStr">
+        <is>
+          <t>PRISIÓN PREVENTIVA OFICIOSA. SU CESE ORDENADO CUANDO EL MINISTERIO PÚBLICO NO PRUEBA NI JUSTIFICA SU PROLONGACIÓN, PARA EFECTOS DE QUE SE DEBATA LA IMPOSICIÓN DE OTRAS MEDIDAS CAUTELARES MENOS RESTRICTIVAS.</t>
+        </is>
+      </c>
+      <c r="L111" s="13" t="inlineStr">
+        <is>
+          <t>2032108</t>
+        </is>
+      </c>
+      <c r="M111" s="13" t="inlineStr"/>
+      <c r="N111" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="O111" s="13" t="inlineStr">
+        <is>
+          <t>SJF 12a Época — VERIFICADO</t>
+        </is>
+      </c>
+      <c r="P111" s="13" t="inlineStr"/>
+      <c r="Q111" s="13" t="inlineStr">
+        <is>
+          <t>Al solicitar prolongación de PPO, el MP tiene carga probatoria. Si no la cumple, el juez debe cesar la PPO y reabrir debate sobre medidas cautelares alternativas.</t>
+        </is>
+      </c>
+      <c r="R111" s="13" t="inlineStr">
+        <is>
+          <t>Defensa decisiva contra prolongación automática de PPO.</t>
+        </is>
+      </c>
+      <c r="S111" s="13" t="inlineStr">
+        <is>
+          <t>Cuando MP solicita prolongación sin justificar, la defensa debe exigir prueba concreta. Sin ella, opera el cese y se debate medida alterna (caución, brazalete, presentación periódica).</t>
+        </is>
+      </c>
+      <c r="T111" s="13" t="inlineStr"/>
+      <c r="U111" s="13" t="inlineStr">
+        <is>
           <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032108</t>
         </is>
       </c>
-      <c r="V108" s="11" t="inlineStr">
+      <c r="V111" s="13" t="inlineStr">
         <is>
           <t>PPO · prolongación · carga probatoria MP · 12a Época</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V108"/>
+  <autoFilter ref="A1:V111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13895,7 +14189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V12"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15068,8 +15362,106 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>auto-2032177</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Responsabilidad administrativa de servidores públicos</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Actualización automática semanal</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Duodécima Época</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>PRUEBAS EN EL JUICIO CONTENCIOSO ADMINISTRATIVO FEDERAL. EL ARTÍCULO 40, PÁRRAFO SEGUNDO, DE LA LEY FEDERAL DE PROCEDIMIENTO CONTENCIOSO ADMINISTRATIVO NO VIOLA EL DERECHO DE ACCESO A LA JUSTICIA.</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>2032177</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr"/>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
+        </is>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>Semanario Judicial de la Federación — captura automática</t>
+        </is>
+      </c>
+      <c r="P13" s="13" t="inlineStr"/>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
+        </is>
+      </c>
+      <c r="R13" s="13" t="inlineStr">
+        <is>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
+        </is>
+      </c>
+      <c r="S13" s="13" t="inlineStr">
+        <is>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="inlineStr"/>
+      <c r="U13" s="13" t="inlineStr">
+        <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032177</t>
+        </is>
+      </c>
+      <c r="V13" s="13" t="inlineStr">
+        <is>
+          <t>Responsabilidad administrativa de servidores públicos · actualización automática</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:V12"/>
+  <autoFilter ref="A1:V13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19571,7 +19963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20935,7 +21327,7 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>amp-gen-001</t>
+          <t>auto-2032154</t>
         </is>
       </c>
       <c r="B15" s="13" t="n">
@@ -20953,12 +21345,12 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Perspectiva de género interseccional</t>
+          <t>Perspectiva de género</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>Acceso a la justicia para mujeres cuidadoras</t>
+          <t>Actualización automática semanal</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
@@ -20983,55 +21375,251 @@
       </c>
       <c r="K15" s="14" t="inlineStr">
         <is>
-          <t>ACCESO A LA JUSTICIA EN CONDICIONES DE IGUALDAD SUSTANTIVA. LAS MANIFESTACIONES DE MUJERES QUE AFIRMAN REALIZAR LABORES DE CUIDADO NO REMUNERADAS DEBEN VALORARSE CON PERSPECTIVA DE GÉNERO INTERSECCIONAL.</t>
+          <t>COMPENSACIÓN ECONÓMICA. ELEMENTOS MÍNIMOS QUE LA PERSONA JUZGADORA DEBE CONSIDERAR PARA MOTIVAR LA RESOLUCIÓN QUE LA CUANTIFICA, CON PERSPECTIVA DE GÉNERO.</t>
         </is>
       </c>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t>2032067</t>
+          <t>2032154</t>
         </is>
       </c>
       <c r="M15" s="13" t="inlineStr"/>
       <c r="N15" s="13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
         </is>
       </c>
       <c r="O15" s="13" t="inlineStr">
         <is>
-          <t>SJF 12a Época — VERIFICADO</t>
+          <t>Semanario Judicial de la Federación — captura automática</t>
         </is>
       </c>
       <c r="P15" s="13" t="inlineStr"/>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>En procesos donde las mujeres afirman dedicarse a labores de cuidado, sus manifestaciones deben valorarse con perspectiva de género interseccional (considerando clase, edad, etnia, discapacidad y otros factores).</t>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
         </is>
       </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
-          <t>Estándar probatorio favorable para mujeres en juicios civiles, familiares, laborales.</t>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
         </is>
       </c>
       <c r="S15" s="13" t="inlineStr">
         <is>
-          <t>En alimentos, pensiones, compensación por trabajo doméstico y otros litigios, el juez debe creer y valorar con flexibilidad las declaraciones de mujeres cuidadoras.</t>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
         </is>
       </c>
       <c r="T15" s="13" t="inlineStr"/>
       <c r="U15" s="13" t="inlineStr">
         <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032154</t>
+        </is>
+      </c>
+      <c r="V15" s="13" t="inlineStr">
+        <is>
+          <t>Perspectiva de género · actualización automática</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>auto-2032184</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Constitucional / DDHH</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Perspectiva de género</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Actualización automática semanal</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Duodécima Época</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>VIOLENCIA FAMILIAR. CUANDO LA VÍCTIMA SEA UNA PERSONA MENOR DE EDAD Y SE ALEGUE ALIENACIÓN O MANIPULACIÓN PARENTAL, EL ÓRGANO JURISDICCIONAL DEBE ORDENAR LA PRÁCTICA DE PRUEBAS PERICIALES PARA VERIFICAR SI SE ACTUALIZA DICHA CONDICIÓN.</t>
+        </is>
+      </c>
+      <c r="L16" s="11" t="inlineStr">
+        <is>
+          <t>2032184</t>
+        </is>
+      </c>
+      <c r="M16" s="11" t="inlineStr"/>
+      <c r="N16" s="11" t="inlineStr">
+        <is>
+          <t>viernes 22 de mayo de 2026 10:27 h</t>
+        </is>
+      </c>
+      <c r="O16" s="11" t="inlineStr">
+        <is>
+          <t>Semanario Judicial de la Federación — captura automática</t>
+        </is>
+      </c>
+      <c r="P16" s="11" t="inlineStr"/>
+      <c r="Q16" s="11" t="inlineStr">
+        <is>
+          <t>Criterio publicado esta semana en el Semanario Judicial de la Federación. Ver texto íntegro en el SJF mediante el enlace directo.</t>
+        </is>
+      </c>
+      <c r="R16" s="11" t="inlineStr">
+        <is>
+          <t>Incorporada automáticamente en la actualización semanal. Pendiente de análisis editorial.</t>
+        </is>
+      </c>
+      <c r="S16" s="11" t="inlineStr">
+        <is>
+          <t>Tesis nueva detectada por el robot semanal. Revisa el texto completo en el SJF.</t>
+        </is>
+      </c>
+      <c r="T16" s="11" t="inlineStr"/>
+      <c r="U16" s="11" t="inlineStr">
+        <is>
+          <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032184</t>
+        </is>
+      </c>
+      <c r="V16" s="11" t="inlineStr">
+        <is>
+          <t>Perspectiva de género · actualización automática</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>amp-gen-001</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Tribunales Colegiados</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Constitucional / DDHH</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Perspectiva de género interseccional</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Acceso a la justicia para mujeres cuidadoras</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>tesis aislada</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Duodécima Época</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>vigente</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>Federal</t>
+        </is>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>ACCESO A LA JUSTICIA EN CONDICIONES DE IGUALDAD SUSTANTIVA. LAS MANIFESTACIONES DE MUJERES QUE AFIRMAN REALIZAR LABORES DE CUIDADO NO REMUNERADAS DEBEN VALORARSE CON PERSPECTIVA DE GÉNERO INTERSECCIONAL.</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>2032067</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr"/>
+      <c r="N17" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>SJF 12a Época — VERIFICADO</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr"/>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>En procesos donde las mujeres afirman dedicarse a labores de cuidado, sus manifestaciones deben valorarse con perspectiva de género interseccional (considerando clase, edad, etnia, discapacidad y otros factores).</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>Estándar probatorio favorable para mujeres en juicios civiles, familiares, laborales.</t>
+        </is>
+      </c>
+      <c r="S17" s="13" t="inlineStr">
+        <is>
+          <t>En alimentos, pensiones, compensación por trabajo doméstico y otros litigios, el juez debe creer y valorar con flexibilidad las declaraciones de mujeres cuidadoras.</t>
+        </is>
+      </c>
+      <c r="T17" s="13" t="inlineStr"/>
+      <c r="U17" s="13" t="inlineStr">
+        <is>
           <t>https://sjf2.scjn.gob.mx/detalle/tesis/2032067</t>
         </is>
       </c>
-      <c r="V15" s="13" t="inlineStr">
+      <c r="V17" s="13" t="inlineStr">
         <is>
           <t>perspectiva género · interseccional · acceso justicia · 12a Época</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V15"/>
+  <autoFilter ref="A1:V17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>